<commit_message>
test(L2): 通し D (J45–J48) の本番実走結果 (58 行: PASS 16 / FAIL 14 / BLOCKED 28) と証拠、workbook 集約 (315/315 行判定済)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/apps/web/.qa/e2e-journey/journey-20260903.xlsx
+++ b/apps/web/.qa/e2e-journey/journey-20260903.xlsx
@@ -7932,14 +7932,25 @@
           <t>「準備中」列に出る。依存・受入基準・仕様書がリンクされて記録される</t>
         </is>
       </c>
-      <c r="K114" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-01.png</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI「タスクを追加」→ POST /tasks 201、lifecycle=triage で画面の「準備中」列に出る (一覧 0→1)。しかしモーダルの入力は タイトル/分類 (機能グループ)/見積 (時間)/種別
+feature
+screen
+foundation
+verification
+infrastructure
+migration/対象画面 (任意 — 例: ログイン画面) だけで、依存・受入基準・仕様書を指定する欄が無く、作成されたタスクは dependencies=[]・acceptance_criteria_id=null・仕様書リンク無し (画面名を入れたのでモック QA-D LP トップ には紐づく)。期待の「依存・受入基準・仕様書がリンクされて記録される」が満たされない。監査: dashboard recent_activities に task.create:task:d01024c7</t>
         </is>
       </c>
     </row>
@@ -7992,14 +8003,19 @@
           <t>依存漏れとして警告が出る。保存する場合も警告つきの状態が記録され、黙って通らない</t>
         </is>
       </c>
-      <c r="K115" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K115" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-02.png</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期待: 依存漏れの警告が出て、保存時も警告つきで記録される / 実測: 「タスクを追加」モーダルに依存を入力する欄が無く (0 個)、依存空のまま保存 → POST /tasks 201 で黙って通る (画面の警告 0 件、カードにも警告表記なし、task.dependencies=[]・metadata/blocked_reason に警告の記録なし)</t>
         </is>
       </c>
     </row>
@@ -8052,14 +8068,20 @@
           <t>受入基準 (3 層) と関連資料が出て、リンク先が実在する。0 件のタブは 0 件の状態で出る</t>
         </is>
       </c>
-      <c r="K116" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K116" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-03.png</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>タブ 受入条件/進捗・スコア/依存タスク/テスト結果/実行履歴/関連資料
+1/コメント。受入条件: GET /acceptance-criteria 404 → 画面「受入条件は登録されていません。」(手動作成タスクには 3 層の受入基準が無く 0 件表示); 関連資料: GET /related 1 件 (設計モック QA-D LP トップ) でリンク先実在= GET /mocks 200; 依存/テスト結果/実行履歴は 0 件の状態で表示 (エラーのタブ 0 件)。「受入基準 (3 層) が出て仕様書が実在」はタスク分解 (AI/Bridge) で作られたタスクでしか検証できない / 解除条件: Mac の Bridge でタスク分解を流す</t>
         </is>
       </c>
     </row>
@@ -8112,14 +8134,19 @@
           <t>列移動が DB に反映され、監査ログ task_status_changed が記録される</t>
         </is>
       </c>
-      <c r="K117" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-04.png</t>
         </is>
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>S-I01 のカードはドラッグ不可 (draggable=false、dragTo でも lifecycle 不変) で、列移動はカードの「着手可にする」ボタン → PATCH /tasks/{id} lifecycle_stage=ready 200。DB 再取得 lifecycle=ready、画面の列=着手可。監査: dashboard recent_activities に task.update:task:d01024c7 (期待の task_status_changed に相当する action 名かは要確認)</t>
         </is>
       </c>
     </row>
@@ -8172,14 +8199,19 @@
           <t>コメントが一覧に出て、担当 AI 社員に通知される (実送信できない環境では送信ログ/キュー投入で代替)</t>
         </is>
       </c>
-      <c r="K118" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K118" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-05.png</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI でコメント投稿 → POST /comments 201 (target_type=task)、GET /comments 1 件、画面のコメント一覧に本文が出る。期待の「担当 AI 社員に通知される (送信ログ/キュー投入)」は通知処理・送信ログ・キューが存在せず観測できない (J46-03/J45-09 と同じ) → 通知部分が不成立</t>
         </is>
       </c>
     </row>
@@ -8232,14 +8264,19 @@
           <t>一覧から消え論理削除が記録される。依存していたタスクに警告が反映される</t>
         </is>
       </c>
-      <c r="K119" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K119" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-20.png</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>S-I01/S-I02 に削除導線が無く (詳細画面の削除ボタン 0 個) API DELETE /tasks/{id} → 204、一覧 5→4・画面から消える・GET 404 (論理削除)、監査 task.delete:task:756ed526。「依存していたタスクに警告」は依存を設定する API/画面が無く依存関係を作れないため未検証 / 解除条件: dependencies を持つタスク (タスク分解 = Bridge) を用意する</t>
         </is>
       </c>
     </row>
@@ -8292,14 +8329,19 @@
           <t>選んだ分だけ着手可に遷移し、選んでいないものは変わらない</t>
         </is>
       </c>
-      <c r="K120" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K120" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-21.png</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期待: 2 件選んで一括操作で選んだ分だけ着手可に遷移 / 実測: S-I01 の選択チェックボックスは着手可 (ready) のカードにしか無く (準備中のカード D/E は選択不可: チェックボックスは Nebula-1・Nebula-3 のみ)、選択バーの操作も「選択を再生する」だけで一括「着手可」は無い。準備中→着手可はカード単体の「着手可にする」を 1 枚ずつ押すしかない。API POST /tasks/bulk/lifecycle (task_ids 2 件, ready) → 200 updated=2 skipped=[] で D/E=ready・選ばなかった F=triage (不変)、画面の列も D/E=着手可 F=準備中、監査 task.bulk_lifecycle 2 件 — データ層は正しいが画面から一括着手可はできない</t>
         </is>
       </c>
     </row>
@@ -8549,14 +8591,19 @@
           <t>工程ごとの成果物が一覧に出て、三層がそれぞれ表示された状態になる</t>
         </is>
       </c>
-      <c r="K124" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K124" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-01.png</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期待: 工程ごとの成果物が一覧に出て三層 (HTML/JSON/MD) が表示される / 実測: GET /outputs 4 件 (estimate/hearing/requirements/verification)。工程画面 S-F01 の成果物欄はどの工程を選んでも同じ 4 件・「成果物 4」で工程ごとに分かれていない。ビューア S-G01 の表示形式タブは実在 format のみで import 成果物は「HTML」だけ (JSON/MD は AI 生成でしか作れず未検証)。しかも HTML 層は content-url が http:// を返すため Mixed Content でブラウザに block され iframe が空 (描画されない)。加えて HTML 成果物で「表を読み込めませんでした。」が常時表示</t>
         </is>
       </c>
     </row>
@@ -8609,14 +8656,19 @@
           <t>署名付き URL (content-url) で HTML が iframe に反映される。Storage に実体が存在する (G-11)</t>
         </is>
       </c>
-      <c r="K125" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K125" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-02.png</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期待: 署名付き URL (content-url) で HTML が iframe に反映され Storage に実体がある / 実測: GET /outputs/{id}/content-url?format=html → 200 で署名付き URL (exp+sig)、直接 fetch → 200 text/html 438 bytes・本文一致 (実体は DB 内蔵 mockdb = G-11 実在)、署名改ざん → 403。しかし URL のスキームが http:// のため https の画面で iframe が Mixed Content として block され、プレビューは空のまま (console: This request has been blocked; the content must be served over HTTPS)</t>
         </is>
       </c>
     </row>
@@ -8670,14 +8722,19 @@
           <t>コメントが一覧に出て、担当 AI 社員にメール通知される (実送信できない環境では送信ログ/キュー投入で代替)。監査ログ comment_created が記録される</t>
         </is>
       </c>
-      <c r="K126" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K126" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-03.png</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI: 対象位置に「2. 機能一覧」(sec-2) を選び投稿 → POST /comments 201、GET /comments に target_element_id=sec-2 で 1 件、画面のコメント一覧に本文表示、unresolved-count 0→undefined。期待の「担当 AI 社員にメール通知 (送信ログ/キュー)」は通知の実装・送信ログ・キューが存在せず観測できない (API 応答にも通知の痕跡なし) → 通知部分が不成立。監査ログ comment_created は運営 API のみで観測不能</t>
         </is>
       </c>
     </row>
@@ -8730,14 +8787,19 @@
           <t>解決済みに遷移し、ダッシュボードの未解決件数が 1 減る</t>
         </is>
       </c>
-      <c r="K127" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K127" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-04.png</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI「解決にする」→ PATCH /comments/{id} 200 status=resolved; ダッシュボード S-B02 (/projects/dashboard) の「未解決コメント」が 1→0 に減る (再読込で実測); GET /comments/unresolved-count も count=0</t>
         </is>
       </c>
     </row>
@@ -8790,14 +8852,19 @@
           <t>提案が一覧に出る。文書はまだ変わらない状態である</t>
         </is>
       </c>
-      <c r="K128" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K128" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-05.png</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: POST /comments/{id}/fix-proposal → 503 (お使いの PC の Bridge がオフラインです。Bridge アプリを起動してから、もう一度お試しください。)、GET /fix-proposals=0 件で文書は不変。UI の「スティーブに修正提案を依頼」は押しても API 呼出が発生しなかった (解決済みコメントのため無効化の可能性)。AI 実行経路 (Bridge/LLM) が無い / 解除条件: Mac の Bridge を接続して再実行</t>
         </is>
       </c>
     </row>
@@ -8850,14 +8917,19 @@
           <t>提案を適用した新版が生成され、版履歴が 1 増える。旧版は残る</t>
         </is>
       </c>
-      <c r="K129" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K129" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J46-06</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: 承認する提案が作れない (J46-05 が Bridge 要で BLOCKED、GET /fix-proposals=0 件) / 解除条件: J46-05 を Mac の Bridge で流してから</t>
         </is>
       </c>
     </row>
@@ -8910,14 +8982,19 @@
           <t>文書は不変で、却下が記録される</t>
         </is>
       </c>
-      <c r="K130" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K130" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J46-07</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>却下する提案が作れない (J46-05 が Bridge 要で BLOCKED、GET /fix-proposals=0 件)。却下 API (POST /output-fix-proposals/{id}/reject) 自体は提案 id が無く叩けない / 解除条件: J46-05 を Mac の Bridge で流してから</t>
         </is>
       </c>
     </row>
@@ -8970,14 +9047,19 @@
           <t>新版が積まれ、一覧の最新版が切り替わる。旧版は履歴に残る</t>
         </is>
       </c>
-      <c r="K131" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K131" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J46-08</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: 「編集」→ POST /outputs/{id}/revise は 503 (お使いの PC の Bridge がオフラインです。Bridge アプリを起動してから、もう一度お試しください。) で AI 実行経路が無い / 解除条件: Mac の Bridge (T-F-41) を接続して再実行。以降の版履歴・差分・復元の行は import で v2 を積んで流す</t>
         </is>
       </c>
     </row>
@@ -9031,14 +9113,19 @@
           <t>版間の差分が表示され、変更箇所が依頼内容と一致して反映される</t>
         </is>
       </c>
-      <c r="K132" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K132" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-09.png</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>版履歴: バージョン選択に 2 版 (v2 · 2026-09-03 05:49 / v1 · 2026-09-03 05:34); 「v1 との差分」→ GET /outputs/{v2}/diff/{v1} 200、画面に unified diff が出て追加行は F-3 レポート出力の 1 行のみ (削除行 1)。ただし v2 は AI 改訂 (J46-08, Bridge 要) ではなく import で積んだため「変更箇所が依頼内容と一致」の AI 側は未検証 / 解除条件: Mac の Bridge で J46-08 を流す</t>
         </is>
       </c>
     </row>
@@ -9091,14 +9178,19 @@
           <t>旧版が新版として復元され、履歴は消えない (版が 1 増える)</t>
         </is>
       </c>
-      <c r="K133" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K133" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-10.png</t>
         </is>
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>v1 を選んで「この版を復元」→ POST /outputs/{v1}/restore 201、v3 が新版として追加 (meta author=restore restored_from_version=1)、履歴は 2→3 版で v1/v2 は消えない、復元版の本文は v1 と同じ (F-3 なし)</t>
         </is>
       </c>
     </row>
@@ -9152,14 +9244,19 @@
           <t>表として出る。編集が新版として保存され、元の版は残る</t>
         </is>
       </c>
-      <c r="K134" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K134" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-11.png</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>S-G01 の「表の表示と編集」に xlsx (見積明細 4 行) が表として出る; セル (設計/単価) 300000→350000 に直して保存 → POST /sheet 201; 版 1→2 (v2 新規)、新版の値=350000、v1 は 300000 のまま残る</t>
         </is>
       </c>
     </row>
@@ -9212,14 +9309,19 @@
           <t>期限つきリンクが 1 度だけ表示され、一覧に出る (URL は再取得不可)。監査ログに記録される</t>
         </is>
       </c>
-      <c r="K135" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K135" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-13.png</t>
         </is>
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI: 期限 30 日を選び「共有リンクを発行」→ POST /outputs/{id}/share-links 201 (expires_at=2026-10-03)、URL が発行直後の画面に 1 度だけ表示、再読込後は URL が消え一覧 (期限・閲覧回数・無効化) だけ残る、GET /share-links の応答に share_url/token 無し (再取得不可)。監査ログ output.share_link.create は運営 API のみで観測不能。所見: 返る share_url が http:// スキーム (クライアントに渡す URL として要確認)</t>
         </is>
       </c>
     </row>
@@ -9272,14 +9374,19 @@
           <t>認証なしで成果物が読める状態になる。期限を過ぎたリンクは拒否される</t>
         </is>
       </c>
-      <c r="K136" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K136" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-14.png</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>認証なし (cookie 0) の別 context で share_url (https) → 200 text/html、成果物本文「要件定義書 QA-D / 1. 目的」が読める、印刷→PDF 導線あり、view_count=1 に反映、不正トークン → 404。「期限を過ぎたリンクは拒否される」は期限切れリンクを作れない (expires_days は最小 1 日: 0 指定 → 422) ため未検証 / 解除条件: staging で expires_at を過去に書き換える手段、または 1 日待つ。所見: API が返す share_url は http:// スキーム</t>
         </is>
       </c>
     </row>
@@ -9333,14 +9440,25 @@
           <t>以後の閲覧は 410 で見えなくなる。無効化の直後 (0 秒) でも見えない (G-12)</t>
         </is>
       </c>
-      <c r="K137" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K137" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-15.png</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI「この共有リンクを無効化」→ POST revoke 200、無効化後の GET /share/{token} → 410; API で発行→GET 200→revoke→応答直後 (0 秒) の GET → 410 (G-12 OK); 二重 revoke → 404; 画面の一覧から消える (「クライアントに渡す
+期限
+7 日
+14 日
+30 日
+90 日
+共有リンクを発行」)</t>
         </is>
       </c>
     </row>
@@ -9393,14 +9511,19 @@
           <t>ファイルが得られ、監査ログ output_downloaded が記録される</t>
         </is>
       </c>
-      <c r="K138" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-16.png</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>API (Bearer) では html (text/html attachment) / xlsx (application/vnd.openxmlformats-officedoc attachment) が得られる。しかし画面の「HTML で保存」「Excel で保存」は API への素の &lt;a href&gt; で Authorization が付かず、クリック結果=HTML で保存: HTTP 404 → 遷移先 /outputs/90f5fb07-96af-4b90-8259-e37315d8c43c/export?format=html 「メインコンテンツへスキップ ワークスペース · QA-D WS 20260903 プロジェクト AI社員 ナレッジ テン」 / Excel で保存: HTTP 404 → 遷移先 /outputs/90f5fb07-96af-4b90-8259-e37315d8c43c/export?format=xlsx 「メインコンテンツへスキップ ワークスペース · QA-D WS 20260903 プロジェクト AI社員 ナレッジ テン」 (画面からはファイルが得られない)。監査ログ output_downloaded は export_output に監査書込が無く記録されない</t>
         </is>
       </c>
     </row>
@@ -9454,14 +9577,19 @@
           <t>編集が DB に反映され updated_at が更新される。次のチャット応答が最新の本文を前提にする</t>
         </is>
       </c>
-      <c r="K139" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K139" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-17.png</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>場所=mac / F-009</t>
+          <t>場所=mac: S-G01 の「編集」は「スティーブに修正を依頼」(POST /revise = AI) のみで、HTML 本文を人が直接編集して保存する UI/API は無い (contenteditable 0 個)。表 (xlsx) の直接編集は J46-11 で PASS。「次のチャット応答が最新の本文を前提にする」はチャット (Bridge) 要 / 解除条件: Mac の Bridge + HTML 直接編集の導線</t>
         </is>
       </c>
     </row>
@@ -9514,14 +9642,19 @@
           <t>403 で拒否され、成果物は変わらない。閲覧とコメントはできる状態である</t>
         </is>
       </c>
-      <c r="K140" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K140" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-18.png</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期待: 403 で拒否 / 実測: viewer (PATCH role=viewer 200) の GET /outputs 200・POST /comments 201 (閲覧・コメント可) は期待通り。編集系は POST /sheet → [500, 500, 500] (恒常 500: サーバー側で問題が発生しました。時間をおいて、もう一度お試しください。（参照 ID: 1d80d498-50fc-4b13-8253-3ff52d9c7268）)、POST /restore → [500, 500, 500] (恒常 500)、POST /revise → 503 (Bridge)、POST /share-links → 201 ×2 (閲覧者がクライアント共有リンクを発行できてしまう = 権限漏れ)。成果物自体は不変 (版数 xlsx=2 req=3)。画面でも編集/共有リンク発行/投稿ボタンが閲覧者に表示される</t>
         </is>
       </c>
     </row>
@@ -9574,14 +9707,19 @@
           <t>0 件の案内が出る状態になり、エラーにならない</t>
         </is>
       </c>
-      <c r="K141" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K141" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-19.png</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>期待: 0 件の案内が出てエラーにならない / 実測: GET /outputs=0 件。S-G01 (/outputs?project=空案件) は「成果物を選択すると表示します。」と出るだけで、成果物を選ぶ一覧・ピッカーが無く 0 件であることも案内しない (件数に関係なく同じ文言)。工程画面 S-F01 側は「成果物 0」と表示。alert 0 件・API エラー無し (JS console の 500 は GET /me/consents の初回 500 = 環境要因)</t>
         </is>
       </c>
     </row>
@@ -9699,14 +9837,19 @@
           <t>生成したモックが一覧に出て、版 v1 が記録される。Storage に HTML の実体がある (G-11)</t>
         </is>
       </c>
-      <c r="K143" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K143" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-01.png</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: UI「新規生成」→ POST /mocks/generate 503 (お使いの PC の Bridge がオフラインです。Bridge アプリを起動してから、もう一度お試しください。)、一覧は 1 件のまま。AI 実行経路 (Bridge) が無い / 解除条件: Mac の Bridge を接続。以降の行は import (GAP-156) で取り込んだモック「QA-D LP トップ」v1 (mockdb 実体あり) で流す</t>
         </is>
       </c>
     </row>
@@ -9759,14 +9902,19 @@
           <t>画面ごとの最新版がプレビューに反映される (署名付き URL)</t>
         </is>
       </c>
-      <c r="K144" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K144" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-02.png</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>一覧のカードから選ぶ → /mocks?mock={id} → GET /mocks/{id}/content-url 200 (署名付き、実体 mockdb は https で直接取得 → 200 本文一致)。しかし URL が http:// スキームのため https の画面で iframe が Mixed Content として block (console 1 件、iframe 本文空) → プレビューに最新版が反映されない (J46-02 と同根)</t>
         </is>
       </c>
     </row>
@@ -9819,14 +9967,19 @@
           <t>切り替えた幅がプレビューに反映された状態になる</t>
         </is>
       </c>
-      <c r="K145" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K145" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-03.png</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>ビューポート切替 (ワイド 1440 / デスクトップ 1024 / タブレット 768 / モバイル 320) を押すと iframe の幅 (style width) が 1440px/1024px/768px/320px に切り替わり aria-pressed も追従。表示上は 752px/752px/752px/320px で、1440/1024/768 は transform scale による fit ズーム で収めている (中身は Mixed Content で空)</t>
         </is>
       </c>
     </row>
@@ -9879,14 +10032,19 @@
           <t>進行状況がストリームで出る。新版が積まれ旧版は残る。一覧の最新版が切り替わる</t>
         </is>
       </c>
-      <c r="K146" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K146" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-04.png</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: UI「修正依頼」→ POST /mocks/{id}/revise/stream は SSE 200 で stage=loading → generating(provider=relay) → error code=bridge_offline「お使いの PC の Bridge がオフライン」で終了、画面に接続手順の案内、版は v1 のまま (新版なし)。AI 実行経路 (Bridge) が無い / 解除条件: Mac の Bridge を接続して再実行</t>
         </is>
       </c>
     </row>
@@ -9939,14 +10097,19 @@
           <t>差分に指示した箇所だけが出る。指示していない作り込みは旧版のまま残る</t>
         </is>
       </c>
-      <c r="K147" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K147" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-05.png</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>場所=cloud / GAP-147 回帰</t>
+          <t>版履歴の「v2 と表示中バージョンの差分」→ GET /mocks/{v3}/diff/{v2} 200、差分は hero-sub の 1 行 (+「商談を一画面で、迷わず。」/ −「商談を一画面で。」) だけで他の作り込みは旧版のまま (追加 1 行・削除 1 行)。ただし v3 は AI 改訂 (J45-04, Bridge 要) ではなく import で積んだため GAP-147 回帰 (AI が指示外を書き換えない) の本体は未検証 / 解除条件: Mac の Bridge で J45-04 を流す</t>
         </is>
       </c>
     </row>
@@ -9999,14 +10162,19 @@
           <t>複製版が履歴に増える</t>
         </is>
       </c>
-      <c r="K148" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K148" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-06.png</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>「…」相当のバージョン一覧メニューから「v1 を複製」→ POST /mocks/{id}/duplicate 201、v2 (meta duplicated_from_version=1) が履歴に増える (1→2)、画面のバージョン一覧にも v2 が出る</t>
         </is>
       </c>
     </row>
@@ -10060,14 +10228,19 @@
           <t>複製版は履歴から消える。唯一の版は 409 で拒否され、残る</t>
         </is>
       </c>
-      <c r="K149" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K149" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-07.png</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>複製版 v2 を「破棄」→「破棄を確定」(2 段階) → POST /mocks/{v2}/discard 200、履歴 2→1 で v2 が消える。残った唯一の版 v3 を同様に破棄 → POST 409 (確定済みのフェーズの成果物は変更できません。追加や修正は次のフェーズで行ってください。)、画面に「確定済みのフェーズの成果物は変更できません。追加や修正は次のフェーズで行ってください。」、v3 は残る (履歴 1 件・GET 200)。所見: 唯一の版の 409 メッセージが「確定済みのフェーズの成果物は変更できません」になっている (フェーズ1 は active。routes/mocks discard_mock_version が ValueError=唯一版 と MockPhaseFrozen を同じ文言に丸めている) — 理由が誤って伝わる</t>
         </is>
       </c>
     </row>
@@ -10121,14 +10294,19 @@
           <t>保存内容が反映されて残る。次のモック生成の前提として使われる</t>
         </is>
       </c>
-      <c r="K150" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K150" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-08.png</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>デザインノートに本文を書いて保存 → PUT /projects/{id}/design-note 200、再読み込み後も同じ本文が欄に残り GET /design-note も一致。「次のモック生成の前提として使われる」は生成が Bridge 要で未検証</t>
         </is>
       </c>
     </row>
@@ -10182,14 +10360,19 @@
           <t>コメントが一覧に出て担当 AI 社員に通知される (実送信できない環境では送信ログ/キュー投入で代替)。解決で状態が遷移する</t>
         </is>
       </c>
-      <c r="K151" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K151" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-09.png</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI でコメント投稿 → POST /comments 201 (target_type=mock)、画面のコメント一覧に出る; 「解決」→ PATCH 200 status=resolved、unresolved-count 2→1 (状態遷移は OK)。期待の「担当 AI 社員に通知される (送信ログ/キュー)」は通知処理・送信ログ・キューが存在せず観測できない (J46-03 と同じ) → 通知部分が不成立</t>
         </is>
       </c>
     </row>
@@ -10242,14 +10425,19 @@
           <t>フェーズごとの最新版だけが一覧に出る状態になる</t>
         </is>
       </c>
-      <c r="K152" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K152" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-10.png</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>フェーズ1 を確定 (confirm 無し → 403 / confirm=true → 200) → フェーズ2 が active。フェーズ2 で import (v4) と複製 (v5) を積む。GET /mocks: delivery_phase_id=phase1 → v3 のみ / phase2 → v4,v5。画面: 既定 (フェーズ2) の一覧は「QA-D LP トップ v5」1 枚だけ、ヘッダーのフェーズ切替 (aria-label フェーズ切替（表示中: フェーズ2）) の一覧「フェーズ1 ✓確定済み 成果物7・モック1」を選ぶと一覧は「QA-D LP トップ v3」1 枚 + 「確定のスナップショットを表示中」表示 (GET /mocks?delivery_phase_id=phase1) — フェーズごとの最新版だけが出る</t>
         </is>
       </c>
     </row>
@@ -10302,14 +10490,19 @@
           <t>拒否され、新版が増えない (凍結が守られる)</t>
         </is>
       </c>
-      <c r="K153" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K153" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-11.png</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>凍結フェーズのモック v3 への POST /revise → 409 (確定済みのフェーズの成果物は変更できません。追加や修正は次のフェーズで行ってください。)、POST /discard → 409、POST /duplicate → 201 (複製は active フェーズ 2 に積まれる); 版数 2→3。UI: 修正依頼 → SSE 200 phase_frozen、alert=「修正依頼に失敗しました。時間をおいて再度お試しください。」。所見: UI の修正依頼 (SSE) は error.code=phase_frozen とメッセージ「「フェーズ1」は確定済みのため変更できません」を受け取っているのに、画面の alert は汎用の「修正依頼に失敗しました。時間をおいて再度お試しください。」で理由を出さない (再試行を促すのは誤誘導)。入力欄も凍結フェーズで disabled になっていない</t>
         </is>
       </c>
     </row>
@@ -11869,14 +12062,19 @@
           <t>ドラフトが一覧に出て、参照したナレッジと生成トレースが記録される</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K177" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-01.png</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: UI「トニーにドラフト生成を依頼」→ POST /sales-docs/generate 503 (お使いの PC の Bridge がオフラインです。Bridge アプリを起動してから、もう一度お試しください。)。AI 実行経路 (Bridge) が無く、依存 J35-01 (ナレッジ) も担当外 / 解除条件: Mac の Bridge を接続して再実行</t>
         </is>
       </c>
     </row>
@@ -11930,14 +12128,19 @@
           <t>一覧に出て、編集が反映される</t>
         </is>
       </c>
-      <c r="K178" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K178" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-02.png</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>種別=見積書で「AI を使わず保存」→ POST /sales-docs 201 (v3)、保存済み一覧 2→3 件・画面に出る; 「編集」→ 設計 300,000→350,000 / 合計 1,900,000→1,950,000 に直して「保存」→ PATCH 200、再取得 summary とプレビューに反映</t>
         </is>
       </c>
     </row>
@@ -11990,14 +12193,19 @@
           <t>PDF が得られ、内容が編集後の状態と一致する</t>
         </is>
       </c>
-      <c r="K179" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K179" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-03.png</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI「PDF」→ GET /sales-docs/{id}/pdf 200 で blob DL (sales-doc-d5961cf2.pdf 2725 bytes)、API でも 200 application/pdf attachment (UI DL と同一テキスト=True)。PDF 本文 (CID フォント HeiseiKakuGo-W5 / UniJIS-UCS2-H) を復号すると「設計 350,000 円」「合計 1,950,000 円」があり、旧値 300,000 は無い = 編集後の状態と一致</t>
         </is>
       </c>
     </row>
@@ -12051,14 +12259,19 @@
           <t>dry_run では実送信せず送信履歴に dry_run と記録される。本送信ではクライアントにメールが届く (実送信できない環境では送信ログ/キュー投入で代替)</t>
         </is>
       </c>
-      <c r="K180" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K180" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-04.png</t>
         </is>
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>dry_run: 宛先 qa-jD-20260903-1@example.com で「クライアントにメール送信」→ POST /sales-docs/{id}/send 201 dry_run=true、送信履歴に dry_run=true で記録され画面にも「dry-run（メール未設定）」バッジ (実送信しない・偽装しない = OK)。本送信: 本番環境にメール送信 (Resend) が未設定のため dry_run にしかならず、本送信は不可 / 解除条件: 本番/staging にメール送信プロバイダを設定 (G-11: 外部リソース未プロビジョニング)。所見: 送信ダイアログにも API にも dry_run/本送信を利用者が選び分ける手段は無く (dry_run はサーバーがメール設定の有無で決める)、正本の「dry_run で送信 → 本送信」の操作列と設計が食い違う</t>
         </is>
       </c>
     </row>
@@ -12111,14 +12324,19 @@
           <t>宛先・日時・dry_run の別が一覧に出る</t>
         </is>
       </c>
-      <c r="K181" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K181" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-05.png</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>GET /sales-docs/{id}/sends 1 件 (to_email・created_at・dry_run=true)、画面の送信履歴カードに宛先・日時・「dry-run（メール未設定）」バッジ が出る</t>
         </is>
       </c>
     </row>
@@ -12171,14 +12389,19 @@
           <t>日本語のエラーで拒否され、送信履歴に増えない</t>
         </is>
       </c>
-      <c r="K182" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K182" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-06.png</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI: 宛先 not-an-email で送信 → 画面側 (input type=email のブラウザ標準検証) で止まり POST は飛ばない。アプリ自身のエラー文言は無く、表示されるのはブラウザ UI 言語の既定文 (本環境では英語「Please include an '@' in the email address.」— 日本語 Chrome なら日本語)。API 直叩き: 'not-an-email' → 422「送信内容を確認してください（入力内容: 形式が正しくありません）。」、'foo@' → 422。送信履歴 1→1 (増えない)。期待の「日本語のエラーで拒否」はアプリの文言としては出ない</t>
         </is>
       </c>
     </row>
@@ -12231,14 +12454,19 @@
           <t>一覧から消え、論理削除が記録される。送信履歴は残る</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K183" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-07.png</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>場所=cloud</t>
+          <t>UI「v3 を削除」→ 確認 → DELETE /sales-docs/{id} 204、一覧 3→2 件・画面から消える、GET detail 404。送信履歴は削除後 GET /sales-docs/{id}/sends → 404 (ドラフトが不可視になると履歴も API/画面から辿れない — DB の行は残るが観測できない)。論理削除の監査は運営 API のみで観測不能</t>
         </is>
       </c>
     </row>
@@ -14910,14 +15138,19 @@
           <t>着手可から実装中に遷移し、Bridge で worker が起動して実行モニター (S-I03) に出る。監査ログ execution_started が記録される</t>
         </is>
       </c>
-      <c r="K224" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K224" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-06.png</t>
         </is>
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: 「再生」→ POST /tasks/{id}/play 202、タスクは lifecycle=in_progress / dispatch_status=queued で投入され executions に 1 件 (running)、監査 task.play:task:d01024c7。Bridge の worker 起動・実行モニター表示は Bridge が無く未検証 / 解除条件: Mac の Bridge を接続</t>
         </is>
       </c>
     </row>
@@ -15036,14 +15269,19 @@
           <t>ログが逐次流れ、status の変化が画面に反映される</t>
         </is>
       </c>
-      <c r="K226" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K226" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-07</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: Bridge (本人 PC の Claude Code) で worker が起動して初めて成立する行。本環境に Bridge ハーネスが無く、実行 (running) 状態・実行ログ・テスト結果・スコアを作れない / 解除条件: Mac の Bridge を接続して J48-06 から順に流す。補足: 実行モニター S-I03 は開ける (J48-13 参照) がログの逐次表示は実行が無く未検証</t>
         </is>
       </c>
     </row>
@@ -15161,14 +15399,19 @@
           <t>テストケース単位の結果が出て、実行の記録と一致する</t>
         </is>
       </c>
-      <c r="K228" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K228" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-08</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: Bridge (本人 PC の Claude Code) で worker が起動して初めて成立する行。本環境に Bridge ハーネスが無く、実行 (running) 状態・実行ログ・テスト結果・スコアを作れない / 解除条件: Mac の Bridge を接続して J48-06 から順に流す。補足: 手動作成タスクの「テスト結果」タブは 0 件表示 (J48-03)</t>
         </is>
       </c>
     </row>
@@ -15221,14 +15464,19 @@
           <t>承認待ちを経ずに完了に遷移し、監査ログ auto_approved が記録される</t>
         </is>
       </c>
-      <c r="K229" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K229" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-09</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: Bridge (本人 PC の Claude Code) で worker が起動して初めて成立する行。本環境に Bridge ハーネスが無く、実行 (running) 状態・実行ログ・テスト結果・スコアを作れない / 解除条件: Mac の Bridge を接続して J48-06 から順に流す。スコア 95% 以上の自動承認 (auto_approved) は kanban_complete を Bridge が呼ばないと発生しない</t>
         </is>
       </c>
     </row>
@@ -15282,14 +15530,19 @@
           <t>承認待ちに出る。承認で done に遷移し、監査ログ approval_required / inbox_entry_resolved が記録される</t>
         </is>
       </c>
-      <c r="K230" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K230" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-10</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: Bridge (本人 PC の Claude Code) で worker が起動して初めて成立する行。本環境に Bridge ハーネスが無く、実行 (running) 状態・実行ログ・テスト結果・スコアを作れない / 解除条件: Mac の Bridge を接続して J48-06 から順に流す。承認待ち (awaiting) は Bridge の完了報告でしか作れない (PATCH lifecycle_stage で作ると実行スコアが無く承認フローの検証にならない)</t>
         </is>
       </c>
     </row>
@@ -15343,14 +15596,19 @@
           <t>差戻で要対応 (blocked) に遷移し、再試行で着手可へ戻る。retry_count が 1 増えて記録される</t>
         </is>
       </c>
-      <c r="K231" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K231" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-11</t>
         </is>
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: J48-10 (承認待ち) が作れないため差戻・再試行の起点が無い / 解除条件: J48-10 を Mac の Bridge で流す</t>
         </is>
       </c>
     </row>
@@ -15403,14 +15661,19 @@
           <t>自動再実装をせず、人間介入を要求する状態で固定される。監査ログ force_intervention が記録される</t>
         </is>
       </c>
-      <c r="K232" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K232" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-12</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: J48-11 (差戻→再試行) を 4 回起こすには Bridge の実行が要る / 解除条件: J48-11 を Mac の Bridge で流す</t>
         </is>
       </c>
     </row>
@@ -15463,14 +15726,19 @@
           <t>接続中の worker 数と並列枠が実数で反映される。イベント集約に直前の実行が記録されている</t>
         </is>
       </c>
-      <c r="K233" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K233" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-13.png</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: GET /bridge/status = {"running_count":0,"queued_count":1,"completing_count":0,"spawning_count":0,"dead_count_24h":0,"parallel_limit":5,"avail; S-I03 の表示 ["Bridge（あなたの PC で動くデスクトップアプリ）がローカル Claude Code を並列起動し、FastAPI 上のディスパッチャがタスクを差配します。実行は完全","Bridge 未接続","同時実行できる数","同時実行枠が空いたら自動で開始）","並列上限を超えた分は、ここに積まれます"]。worker 接続と直前の実行イベントは Bridge が無く未検証 / 解除条件: Mac の Bridge を接続</t>
         </is>
       </c>
     </row>
@@ -15523,14 +15791,19 @@
           <t>キューから外れ、実行されない状態に戻る</t>
         </is>
       </c>
-      <c r="K234" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K234" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-14.png</t>
         </is>
       </c>
       <c r="M234" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>J48-06 で queued にしたタスクを S-I03 の「キュー取消」 → 200、lifecycle in_progress/queued → ready/null (実行されない状態に戻る)、executions=cancelled</t>
         </is>
       </c>
     </row>
@@ -15583,14 +15856,19 @@
           <t>実行が cancelled で閉じ、席が返る。タスクは要対応として残る</t>
         </is>
       </c>
-      <c r="K235" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K235" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-15</t>
         </is>
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: 実行中 (spawning/running) のセッションは Bridge が無いと作れない。queued 状態で POST /tasks/{id}/dispatch-stop → 409 (いまの状態ではこの操作を行えません。画面を再読み込みしてお試しください。) で「実行中でない」と拒否 (queued は J48-14 のキュー取消で戻す設計)。/ 解除条件: Mac の Bridge で J48-06 を流し running にしてから停止</t>
         </is>
       </c>
     </row>
@@ -15643,14 +15921,19 @@
           <t>次の pick でそのタスクが最優先で実行中に遷移する</t>
         </is>
       </c>
-      <c r="K236" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K236" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-16</t>
         </is>
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: 「順番待ちから 1 件追加」(POST /dispatch/promote) の効果は次の pick (Bridge の kanban.pick) でしか観測できない / 解除条件: Mac の Bridge を接続</t>
         </is>
       </c>
     </row>
@@ -15703,14 +15986,19 @@
           <t>PID ポーリングで検出され、自動で再 spawn される。監査ログ worker_dead_reclaimed が記録される</t>
         </is>
       </c>
-      <c r="K237" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K237" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-18</t>
         </is>
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t>場所=mac / G-15</t>
+          <t>場所=mac / G-15: 実行中の claude プロセスを kill する操作は本人 PC 側 / 解除条件: Mac の Bridge で実行中に kill</t>
         </is>
       </c>
     </row>
@@ -15763,14 +16051,19 @@
           <t>完了扱いにならず、要対応として残る状態になる。空の要約が完了として記録されない</t>
         </is>
       </c>
-      <c r="K238" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K238" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-19</t>
         </is>
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t>場所=mac / G-15</t>
+          <t>場所=mac / G-15: kanban_complete を呼ばず exit 0 する worker は Bridge 側で作る / 解除条件: Mac の Bridge でハーネス worker を用意</t>
         </is>
       </c>
     </row>
@@ -16548,14 +16841,19 @@
           <t>選んだ処理が反映され、確認カードが消える。監査ログ task_paused_for_change が記録される</t>
         </is>
       </c>
-      <c r="K250" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K250" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>journeys-D-prod-20260903.txt#J48-17</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>場所=mac / F-CUC02</t>
+          <t>場所=mac / F-CUC02: 仕様変更の確認カードはチャット (Bridge) で仕様変更を発言し、実行中タスクに紐づくモックの新版が検知されて出る。チャットも実行も Bridge 要 / 解除条件: Mac の Bridge で J41-02 と J48-06 を流す</t>
         </is>
       </c>
     </row>
@@ -16934,14 +17232,19 @@
           <t>本人 PC で修正され、新版として反映される</t>
         </is>
       </c>
-      <c r="K256" s="2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="K256" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-12.png</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>場所=mac</t>
+          <t>場所=mac: UI「AI にファイルごと直してもらう」→ POST /outputs/{id}/ai-file-edit 503 (お使いの PC の Bridge がオフラインです。Bridge アプリを起動してから、もう一度お試しください。)、版は 2 のまま。本人 PC の Bridge が無い / 解除条件: Mac の Bridge を接続して再実行</t>
         </is>
       </c>
     </row>
@@ -21100,11 +21403,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>35%</t>
         </is>
       </c>
     </row>
@@ -21115,11 +21418,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>17%</t>
         </is>
       </c>
     </row>
@@ -21130,11 +21433,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>49%</t>
         </is>
       </c>
     </row>
@@ -21145,11 +21448,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(L2): 通し A〜F 315 行を journey-20260903.xlsx に集約 (PASS 112 / FAIL 49 / BLOCKED 154)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/apps/web/.qa/e2e-journey/journey-20260903.xlsx
+++ b/apps/web/.qa/e2e-journey/journey-20260903.xlsx
@@ -586,19 +586,19 @@
           <t>500 や白画面にならず、各画面が 0 件の状態として表示される。API は空配列を返し、サーバのエラーログに例外が記録されない</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J00-01.png</t>
+          <t>apps/web/.qa/evidence/ps28-30-prod-20260903.txt</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>期待: 500 や白画面にならず各画面が 0 件で表示 / 実測 (前提の「全テーブルを空にする」は本番 DB のため不可 → データ 0 件の新規アカウントで代替): 19 画面とも白画面ではなく 0 件表示だが、9/19 画面で画面が同時に叩く API のどれかが断続的に 500 (参照 ID 付き) を返す: [["/projects/dashboard", ["GET /me/consents 500"]], ["/employees", ["GET /ai-employees 500"]], ["/workflow", ["GET /approval-inbox?status=pending 500"]], ["/knowledge/review", ["GET /approval-inbox?status=pending 500"]], ["/meetings", ["GET /me/consents 500"]], ["/sales", ["GET /me 500"]], ["/chat", ["GET /me 500"]], ["/projects/settings", ["GET /approval-inbox?status=pending 500"]], ["/projects/vault", ["GET /me 500"]]]。同一 API は直列 30 回だと全 200、同時 10 本だと 1〜2 本が 500 (fly-request-id を証拠に記録)。サーバのエラーログは運営画面でしか見られず未観測</t>
+          <t>再測 2026-09-03 07:09: 同時 10 本 × 3 回、直列 20 本、画面相当 6 本同時 × 5 回で 5xx = 0 (旧 FAIL は EMAXCONNSESSION = GAP-291)。空 DB での 19 画面 0 件表示は本番では不可 (前提のデータ 0 件アカウントで代替済み)</t>
         </is>
       </c>
     </row>
@@ -1701,19 +1701,19 @@
           <t>改訂した内容がそのまま反映されて読める。ダミーの連絡先や存在しないプランが残っていない</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J03-02.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J03-02-terms.png</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>期待: 改訂内容がそのまま読める・ダミー連絡先や存在しないプランが残っていない / 実測: 3 ページとも本文が出ず role=alert「文書の取得に失敗しました。時間をおいて再度お試しください。」(画面が叩く GET /public/legal-documents/{type} が全て 500・参照 ID 付き)。認証付き経路 GET /me/consents では legal_documents 2026-08-22 版が読めるので、anon 経路 (set local role anon) 固有の障害 = G-11 (本番 DB の anon ロール/権限) の疑い。文面の内容 (ダミー連絡先の有無) は本文が出ないため未判定</t>
+          <t>再測 2026-09-03 07:15 (実ブラウザ): /terms 4,581 文字 / /privacy 2,464 文字 / /tokushoho 908 文字が「最終更新 2026年8月22日 · バージョン 2026-08-22」つきで表示。取得失敗の帯なし。旧 FAIL は API 500 (GAP-290/291) が原因</t>
         </is>
       </c>
     </row>
@@ -1832,19 +1832,19 @@
           <t>3 種 (規約/プライバシー/特商法) が版番号つきで一覧に出て、未サインインで読める</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J03-04.png</t>
+          <t>apps/web/.qa/evidence/ps28-30-prod-20260903.txt</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>期待: 3 種が版番号つきで一覧に出て未サインインで読める / 実測: GET /public/legal-documents -&gt; 500 サーバー側で問題が発生しました。時間をおいて、もう一度お試しください。（参照 ID: fcf2c584-cb32-4a60-8070-ccc279f3dcc7）; 画面 /terms (S-A01 新規登録タブの「利用規約」リンクから到達) は role=alert「文書の取得に失敗しました。時間をおいて再度お試しください。|利用規約 | Atelier | Atelier」で本文が出ない (画面が叩いた GET /public/legal-documents/terms_of_service -&gt; 500). 版番号=false</t>
+          <t>再測 2026-09-03 07:09 (transaction pooler 切替後): GET /public/legal-documents?locale=ja 200 (21,622 bytes)、terms/privacy/tokushoho 各 200。旧 FAIL の 500 は Session pooler 上限超過 (GAP-291) が原因</t>
         </is>
       </c>
     </row>
@@ -21403,11 +21403,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
@@ -21418,11 +21418,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>16%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(正本): GAP-310/311/312 起票、SE01-902 / SG01-905 / PS-31 追加、通し R2 再測 (17 行: PASS 3 / FAIL 14) を集約
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/apps/web/.qa/e2e-journey/journey-20260903.xlsx
+++ b/apps/web/.qa/e2e-journey/journey-20260903.xlsx
@@ -7939,18 +7939,18 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J48-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-01-r2.png</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>UI「タスクを追加」→ POST /tasks 201、lifecycle=triage で画面の「準備中」列に出る (一覧 0→1)。しかしモーダルの入力は タイトル/分類 (機能グループ)/見積 (時間)/種別
+          <t>[再測 R2] UI「タスクを追加」→ POST /tasks 201、lifecycle=triage で画面の「準備中」列に出る (一覧 0→1)。モーダルの入力は タイトル/分類 (機能グループ)/見積 (時間)/種別
 feature
 screen
 foundation
 verification
 infrastructure
-migration/対象画面 (任意 — 例: ログイン画面) だけで、依存・受入基準・仕様書を指定する欄が無く、作成されたタスクは dependencies=[]・acceptance_criteria_id=null・仕様書リンク無し (画面名を入れたのでモック QA-D LP トップ には紐づく)。期待の「依存・受入基準・仕様書がリンクされて記録される」が満たされない。監査: dashboard recent_activities に task.create:task:d01024c7</t>
+migration/対象画面 (任意 — 例: ログイン画面) で、依存・受入基準・仕様書を指定する欄=0 個。作成されたタスクは dependencies=[]・acceptance_criteria_id=null・仕様書リンク無し (対象画面 → mock_screen_name=QA-R2 LP トップ には紐づく) → 期待の「依存・受入基準・仕様書がリンクされて記録される」が満たされない</t>
         </is>
       </c>
     </row>
@@ -8010,12 +8010,12 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J48-02.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-02-r2.png</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>期待: 依存漏れの警告が出て、保存時も警告つきで記録される / 実測: 「タスクを追加」モーダルに依存を入力する欄が無く (0 個)、依存空のまま保存 → POST /tasks 201 で黙って通る (画面の警告 0 件、カードにも警告表記なし、task.dependencies=[]・metadata/blocked_reason に警告の記録なし)</t>
+          <t>[再測 R2] 期待: 依存漏れの警告が出て、保存時も警告つきで記録される / 実測: 「タスクを追加」モーダルに依存を入力する欄が 0 個、依存空のまま保存 → POST /tasks 201 で黙って通る (画面の警告 0 件、カードに警告表記なし — 前判定の「警告表記=true」は自分で付けたタイトル「Nebula-2 依存なし」が検出語に当たった誤検出、task.dependencies=[]・metadata/blocked_reason に警告の記録なし)。通し D と同じ (GAP-303 未着手)</t>
         </is>
       </c>
     </row>
@@ -8206,12 +8206,12 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J48-05.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-05-r2.png</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>UI でコメント投稿 → POST /comments 201 (target_type=task)、GET /comments 1 件、画面のコメント一覧に本文が出る。期待の「担当 AI 社員に通知される (送信ログ/キュー投入)」は通知処理・送信ログ・キューが存在せず観測できない (J46-03/J45-09 と同じ) → 通知部分が不成立</t>
+          <t>[再測 R2] UI でコメント投稿 → POST /comments 201 (target_type=task)、GET /comments 1 件、画面のコメント一覧に本文が出る。期待の「担当 AI 社員に通知される (送信ログ/キュー投入)」: 通知の痕跡=false (担当社員のスレッド・approval-inbox・dashboard・API 応答のいずれにも通知の痕跡なし → 不成立)</t>
         </is>
       </c>
     </row>
@@ -8336,12 +8336,12 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J48-21.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-21-r2.png</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>期待: 2 件選んで一括操作で選んだ分だけ着手可に遷移 / 実測: S-I01 の選択チェックボックスは着手可 (ready) のカードにしか無く (準備中のカード D/E は選択不可: チェックボックスは Nebula-1・Nebula-3 のみ)、選択バーの操作も「選択を再生する」だけで一括「着手可」は無い。準備中→着手可はカード単体の「着手可にする」を 1 枚ずつ押すしかない。API POST /tasks/bulk/lifecycle (task_ids 2 件, ready) → 200 updated=2 skipped=[] で D/E=ready・選ばなかった F=triage (不変)、画面の列も D/E=着手可 F=準備中、監査 task.bulk_lifecycle 2 件 — データ層は正しいが画面から一括着手可はできない</t>
+          <t>[再測 R2] 期待: 2 件選んで一括操作で選んだ分だけ着手可 / 実測: S-I01 の選択チェックボックスは着手可のカードにしか無く (準備中カード G/H/I には 0 個、check は 2 件とも不可)、選択バーも出ず、選択バー系の一括「着手可にする」ボタンは無い (画面にあるのはカード単体の「…を着手可にする」6 個 = 1 枚ずつ押すしかない。再実行のハーネスが自分のタイトルの「一括」を含むカード単体ボタンを誤って 1 回押した = E を単体で ready にしただけ)。API POST /tasks/bulk/lifecycle (task_ids 2 件, ready) → 200 {"data":{"requested":2,"updated":2,"updated_task_ids":["ee4b6d8a-bd4e-4101-baab-a577413ad382","52a8deff-721b-4cd5-91dd-1 で G/H=ready・選ばなかった I=triage (不変)、画面の列 {"G":"着手可","H":"着手可","I":"準備中"}、監査 task.bulk_lifecycle ["task.bulk_lifecycle:task:52a8deff","task.bulk_lifecycle:task:ee4b6d8a"] — データ層は正しいが画面から一括着手可はできない (GAP-304 未着手・通し D と同じ)</t>
         </is>
       </c>
     </row>
@@ -8598,12 +8598,12 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-01-r2.png</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>期待: 工程ごとの成果物が一覧に出て三層 (HTML/JSON/MD) が表示される / 実測: GET /outputs 4 件 (estimate/hearing/requirements/verification)。工程画面 S-F01 の成果物欄はどの工程を選んでも同じ 4 件・「成果物 4」で工程ごとに分かれていない。ビューア S-G01 の表示形式タブは実在 format のみで import 成果物は「HTML」だけ (JSON/MD は AI 生成でしか作れず未検証)。しかも HTML 層は content-url が http:// を返すため Mixed Content でブラウザに block され iframe が空 (描画されない)。加えて HTML 成果物で「表を読み込めませんでした。」が常時表示</t>
+          <t>[再測 R2] 期待: 工程ごとの成果物が一覧に出て三層 (HTML/JSON/MD) が表示される / 実測: GET /outputs 5 件 (estimate/requirements/verification/hearing)。S-G01 (?output 無し) は「成果物を選択すると表示します」で成果物を選ぶ一覧=0 個。S-F01 工程ごとの成果物欄=["ヒアリング:0件","要件定義:0件","アーキ設計:0件","デザイン:0件","機能分解:0件"] (工程で分かれる=false)。ビューアの表示形式タブ=["HTML"]、HTML 層は iframe 内本文「1. 目的  QA-R2 案件の要件定義書 v1。Nebul」(Mixed Content 0 件)、alert=["この成果物は表形式ではありません。HTML の成果物は本文プレビューで開けます。"]。JSON/MD タブは import 成果物では未生成 (0 個)</t>
         </is>
       </c>
     </row>
@@ -8656,19 +8656,19 @@
           <t>署名付き URL (content-url) で HTML が iframe に反映される。Storage に実体が存在する (G-11)</t>
         </is>
       </c>
-      <c r="K125" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K125" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-02.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-02-r2.png</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>期待: 署名付き URL (content-url) で HTML が iframe に反映され Storage に実体がある / 実測: GET /outputs/{id}/content-url?format=html → 200 で署名付き URL (exp+sig)、直接 fetch → 200 text/html 438 bytes・本文一致 (実体は DB 内蔵 mockdb = G-11 実在)、署名改ざん → 403。しかし URL のスキームが http:// のため https の画面で iframe が Mixed Content として block され、プレビューは空のまま (console: This request has been blocked; the content must be served over HTTPS)</t>
+          <t>[再測 R2] GET content-url?format=html → 200 で https の署名付き URL (exp+sig, expires_at=undefined)、画面の iframe src が同 URL、iframe 内に「1. 目的」が描画 (Mixed Content 0 件)。署名 URL を直接取得 → 200 text/html 440 bytes 本文一致 (実体あり = G-11)、署名改ざん → 403</t>
         </is>
       </c>
     </row>
@@ -8729,12 +8729,12 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-03.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-03-r2.png</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>UI: 対象位置に「2. 機能一覧」(sec-2) を選び投稿 → POST /comments 201、GET /comments に target_element_id=sec-2 で 1 件、画面のコメント一覧に本文表示、unresolved-count 0→undefined。期待の「担当 AI 社員にメール通知 (送信ログ/キュー)」は通知の実装・送信ログ・キューが存在せず観測できない (API 応答にも通知の痕跡なし) → 通知部分が不成立。監査ログ comment_created は運営 API のみで観測不能</t>
+          <t>[再測 R2] UI: 対象位置に「2. 機能一覧」(sec-2) を選び投稿 → POST /comments 201、GET /comments に target_element_id=sec-2 で 1 件、画面のコメント一覧に本文=true、unresolved-count 0→1。期待の「担当 AI 社員にメール通知 (送信ログ/キュー)」: 通知の痕跡=false (API 応答に通知フィールド無し、担当社員のスレッド一覧・approval-inbox・tool-approvals に変化なし = 通知処理・送信ログ・キューが存在せず観測できない → 不成立)。監査 comment_created: dashboard recent_activities に増えた項目=["comment.create:comment:01bde75a"] (comment 対象の監査は運営 API のみで観測不能)</t>
         </is>
       </c>
     </row>
@@ -9518,12 +9518,12 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-16.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-16-r2.png</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>API (Bearer) では html (text/html attachment) / xlsx (application/vnd.openxmlformats-officedoc attachment) が得られる。しかし画面の「HTML で保存」「Excel で保存」は API への素の &lt;a href&gt; で Authorization が付かず、クリック結果=HTML で保存: HTTP 404 → 遷移先 /outputs/90f5fb07-96af-4b90-8259-e37315d8c43c/export?format=html 「メインコンテンツへスキップ ワークスペース · QA-D WS 20260903 プロジェクト AI社員 ナレッジ テン」 / Excel で保存: HTTP 404 → 遷移先 /outputs/90f5fb07-96af-4b90-8259-e37315d8c43c/export?format=xlsx 「メインコンテンツへスキップ ワークスペース · QA-D WS 20260903 プロジェクト AI社員 ナレッジ テン」 (画面からはファイルが得られない)。監査ログ output_downloaded は export_output に監査書込が無く記録されない</t>
+          <t>[再測 R2] 画面の「HTML で保存」「Excel で保存」= HTML で保存: HTTP 404 (Authorization 無し) → 遷移先 /outputs/177da0f1-d3ed-4e95-ba54-bd48b80c7b67/export?format=html 「メインコンテンツへスキップ ワークスペース · QA-R2 WS 2026090」 / Excel で保存: HTTP 404 (Authorization 無し) → 遷移先 /outputs/177da0f1-d3ed-4e95-ba54-bd48b80c7b67/export?format=xlsx 「メインコンテンツへスキップ ワークスペース · QA-R2 WS 2026090」。API (Bearer) は html 200 / xlsx 200 (4987 bytes) で得られる。監査 output_downloaded は dashboard に増えず (["task.create:task:9da8b7d4","task.create:task:22fa0df7"]) 観測できない</t>
         </is>
       </c>
     </row>
@@ -9649,12 +9649,12 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-18.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-18-r2.png</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>期待: 403 で拒否 / 実測: viewer (PATCH role=viewer 200) の GET /outputs 200・POST /comments 201 (閲覧・コメント可) は期待通り。編集系は POST /sheet → [500, 500, 500] (恒常 500: サーバー側で問題が発生しました。時間をおいて、もう一度お試しください。（参照 ID: 1d80d498-50fc-4b13-8253-3ff52d9c7268）)、POST /restore → [500, 500, 500] (恒常 500)、POST /revise → 503 (Bridge)、POST /share-links → 201 ×2 (閲覧者がクライアント共有リンクを発行できてしまう = 権限漏れ)。成果物自体は不変 (版数 xlsx=2 req=3)。画面でも編集/共有リンク発行/投稿ボタンが閲覧者に表示される</t>
+          <t>[再測 R2] 期待: 403 で拒否され成果物は変わらない・閲覧とコメントはできる / 実測: PATCH role=viewer 200。viewer の GET /outputs/{id} 200 (閲覧可)、POST /comments 201 (コメント可) は期待通り。編集系 (各 3 回): POST /sheet [403,403,403]「この操作を行う権限がありません。」(GAP-282 の 500→403 は解消)、POST /share-links [403,403,403]「共有リンクを発行する権限がありません。」(GAP-307 解消)、POST /restore は最新版に対しては [409,409,409]「この版は復元できません」(前提チェックが権限より先) — v2 を import で積んで旧版 v1 に対して試すと [403,403,403] (権限判定は正しい)。POST /revise は [503,503,503]「お使いの PC の Bridge がオフラインです」(Bridge 判定が権限判定より先で、閲覧者にも 403 ではなく 503 が返る = 期待の 403 に不一致)。版数 xlsx 2→2・要件定義 2→3 (増分は対照の owner restore のみ、viewer の操作では不変)。画面: 閲覧者にも「編集 / 新しい版として保存 / AI に修正を依頼 / 共有リンクを発行 / HTML で保存 / Excel で保存 / 投稿」が表示され、「保存」を押すと POST /sheet 403 → alert「保存に失敗しました。」(理由が権限だと分からない)</t>
         </is>
       </c>
     </row>
@@ -9714,12 +9714,12 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-19.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-19-r2.png</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>期待: 0 件の案内が出てエラーにならない / 実測: GET /outputs=0 件。S-G01 (/outputs?project=空案件) は「成果物を選択すると表示します。」と出るだけで、成果物を選ぶ一覧・ピッカーが無く 0 件であることも案内しない (件数に関係なく同じ文言)。工程画面 S-F01 側は「成果物 0」と表示。alert 0 件・API エラー無し (JS console の 500 は GET /me/consents の初回 500 = 環境要因)</t>
+          <t>[再測 R2] 期待: 0 件の案内が出てエラーにならない / 実測: GET /outputs=0 件。S-G01 は「成果物を選択すると表示します」(0 件の案内=false)、alert 0 件、API 5xx=0 件、工程画面の成果物欄=「成果物 0 件)」</t>
         </is>
       </c>
     </row>
@@ -9902,19 +9902,20 @@
           <t>画面ごとの最新版がプレビューに反映される (署名付き URL)</t>
         </is>
       </c>
-      <c r="K144" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K144" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J45-02.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-02-r2.png</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>一覧のカードから選ぶ → /mocks?mock={id} → GET /mocks/{id}/content-url 200 (署名付き、実体 mockdb は https で直接取得 → 200 本文一致)。しかし URL が http:// スキームのため https の画面で iframe が Mixed Content として block (console 1 件、iframe 本文空) → プレビューに最新版が反映されない (J46-02 と同根)</t>
+          <t>[再測 R2] 一覧のカードから選ぶ → /mocks?mock={id} → GET /mocks/{id}/content-url 200 (https の署名付き URL)、iframe に最新版 v1 の本文「Nebula 商談管理
+商談を一画面で」が描画 (Mixed Content 0 件)、署名 URL の直接取得 200 本文一致</t>
         </is>
       </c>
     </row>
@@ -10367,12 +10368,12 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J45-09.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J45-09-r2.png</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>UI でコメント投稿 → POST /comments 201 (target_type=mock)、画面のコメント一覧に出る; 「解決」→ PATCH 200 status=resolved、unresolved-count 2→1 (状態遷移は OK)。期待の「担当 AI 社員に通知される (送信ログ/キュー)」は通知処理・送信ログ・キューが存在せず観測できない (J46-03 と同じ) → 通知部分が不成立</t>
+          <t>[再測 R2] UI でコメント投稿 → POST /comments 201 (target_type=mock)、GET /comments 1 件、画面のコメント一覧に出る、unresolved-count 3→4; 「解決」→ PATCH 200 status=resolved、unresolved-count 4→3 (状態遷移は OK)。期待の「担当 AI 社員に通知される (送信ログ/キュー)」: 通知の痕跡=false (ワンダのスレッド・approval-inbox・dashboard・API 応答のいずれにも通知の痕跡なし → 不成立、GAP-299 未着手)</t>
         </is>
       </c>
     </row>
@@ -12396,12 +12397,12 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J47-06.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-06-r2.png</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>UI: 宛先 not-an-email で送信 → 画面側 (input type=email のブラウザ標準検証) で止まり POST は飛ばない。アプリ自身のエラー文言は無く、表示されるのはブラウザ UI 言語の既定文 (本環境では英語「Please include an '@' in the email address.」— 日本語 Chrome なら日本語)。API 直叩き: 'not-an-email' → 422「送信内容を確認してください（入力内容: 形式が正しくありません）。」、'foo@' → 422。送信履歴 1→1 (増えない)。期待の「日本語のエラーで拒否」はアプリの文言としては出ない</t>
+          <t>[再測 R2] UI: 宛先 'not-an-email' → POST 未送信、アプリのエラー文言=[] (ブラウザ標準の検証のみ: validationMessage「Please include an '@' in the email address. 'not-an-email' is missing an '@'.」= ブラウザ UI 言語依存) / 'foo@' → POST 未送信、アプリのエラー文言=[] (ブラウザ標準の検証のみ: validationMessage「Please enter a part following '@'. 'foo@' is incomplete.」= ブラウザ UI 言語依存); API: 'not-an-email' → 422 "送信内容を確認してください（入力内容: 形式が正しくありません）。"、'foo@' → 422; 送信履歴 1→1 (増えない)</t>
         </is>
       </c>
     </row>
@@ -12461,12 +12462,12 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J47-07.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-07-r2.png</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>UI「v3 を削除」→ 確認 → DELETE /sales-docs/{id} 204、一覧 3→2 件・画面から消える、GET detail 404。送信履歴は削除後 GET /sales-docs/{id}/sends → 404 (ドラフトが不可視になると履歴も API/画面から辿れない — DB の行は残るが観測できない)。論理削除の監査は運営 API のみで観測不能</t>
+          <t>[再測 R2] UI「v2 を削除」→ 確認 → DELETE /sales-docs/{id} 204、一覧 2→1 件・画面から消える、GET detail 404。送信履歴: 削除前 1 件 → 削除後 GET /sales-docs/{id}/sends 404 (ドラフトが不可視になると送信履歴も API/画面から辿れない)。論理削除の監査は運営 API のみで観測不能 (dashboard 増分=["task.update:task:7e00a0ab"])</t>
         </is>
       </c>
     </row>
@@ -12526,12 +12527,12 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J44-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J44-01-r2.png</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>期待: 画面表示が GET /cron-actions と一致 / 実測: 一覧・コストは出るが、作成フォーム (ScheduleBuilder) の種類名・コスト表示は画面側のハードコード (ACTIONS 定数) で、API の title (例 API「タスク自動再生」↔ 画面「着手可のタスクを再生する」) / cost_label (API「本人の Claude プラン枠」「コスト無料」↔ 画面「プラン枠」「無料」) と 6 種中 4 種で文言不一致。GET /cron-actions は取得されるが作成フォームには反映されていない (GAP-179 の「唯一の信頼源」に反する)</t>
+          <t>[再測 R2] 期待: 画面表示が GET /cron-actions と一致 / 実測: 6 種中 欠け 6 ["task_replay","knowledge_organize","industry_extract","report_summary","daily_digest","weekly_burndown"]、旧文言残存 ["着手可のタスクを再生する","ナレッジを整理する","横断パターンを抽出する","プラン枠","無料"]</t>
         </is>
       </c>
     </row>
@@ -15007,19 +15008,19 @@
           <t>raw トークンが 1 度だけ表示され、一覧に出る。再読み込み後は二度と出ない</t>
         </is>
       </c>
-      <c r="K222" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K222" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J40-04.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J40-04-r2.png</t>
         </is>
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>期待: raw が 1 度だけ表示され一覧に出る・再読み込み後は出ない / 実測: UI「接続トークンを発行」→ POST 201 で raw (43 文字) が発行直後の画面に 1 度表示され、再読み込み後は画面に出ず GET /bridge-tokens にも raw 無し (ここは期待通り)。しかし「一覧に出る」が不安定: 発行 3 秒後の GET /bridge-tokens が 200 {data:[]} (発行済みトークンが 0 件) で返り、その後 20 回連続 GET で 2 回 (10%) が 500「サーバー側で問題が発生しました（参照 ID 付き）」。同じ本人・同じ条件で件数 0 / 3 / 500 が揺れる (list_tokens が別プール _service_session を使う経路の不安定さと推定)</t>
+          <t>[再測 R2] UI「接続トークンを発行」→ POST 201、raw (43 文字) が発行直後の画面に 1 度表示。発行直後 0〜3.5 秒の GET /bridge-tokens は全て 200 で発行 id を含み token フィールド無し (4 回)。再読み込み後は raw が画面に出ず、パネルの一覧に発行済みトークン (id/label/日時) が出る。20 回連続 GET の分布 {"200/1件":20} (500 なし・件数の揺れなし)、include_revoked=true → 200</t>
         </is>
       </c>
     </row>
@@ -17895,12 +17896,12 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J43-03.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J43-03-r2.png</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>期待: 送信失敗時に入力欄へ文章が戻り、押し直すだけで再送できる / 実測: Bridge 未接続で送信 → POST /chat/threads/{id}/stream 200 (SSE) → 画面 alert「お使いの PC がまだ接続されていません。設定画面の「Bridge を接続」から接続すると、AI 機能を使えるようになります。」が出るが、入力欄は空に戻り (value="")、文章はユーザー発話として DB に保存されるだけ (GET messages に role=user 1 件・assistant 無し・queued 0 件)。押し直しても送るものが無く再送されない。再現: S-E01 でスレッドを開き、Bridge 未接続のまま文章を入力して送信 → 入力欄が消える</t>
+          <t>[再測 R2] 期待: 入力欄に文章が戻り押し直しで再送 / 実測: 送信 API=POST 200 /chat/threads/3a0342c1-d6b9-467b-a1fc-81c4432c18e8/stream, POST 200 /chat/threads/3a0342c1-d6b9-467b-a1fc-81c4432c18e8/queued/consume、alert=["お使いの PC がまだ接続されていません。設定画面の「Bridge を接続」から接続すると、AI 機能を使えるようになります。"]、入力欄="" (一致=false)、DB messages 1→2、押し直し API=[]</t>
         </is>
       </c>
     </row>
@@ -21403,11 +21404,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>37%</t>
         </is>
       </c>
     </row>
@@ -21418,11 +21419,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>15%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(L2): 通し R1 再測 (31 行: PASS 9 / FAIL 20 / BLOCKED 2) を集約 — 画面側は Vercel 未配信、API 側の残りは GAP-313〜315 へ
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/apps/web/.qa/e2e-journey/journey-20260903.xlsx
+++ b/apps/web/.qa/e2e-journey/journey-20260903.xlsx
@@ -2301,12 +2301,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J10-07.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J10-07-r1.png</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>期待: 日本語エラーで拒否・WS 増えない / 実測: errors=[] native={"noValidate":false,"vm":"","req":false} POST= WS 件数=0</t>
+          <t>[再測 R1] 期待: 日本語エラーで拒否・WS 増えない / 実測: errors=[] POST=未送信 disabled=true WS 件数=0</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3488,12 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J15-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J15-01-r1.png</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>期待: 登録直後に 3 ステップのウォークスルーが出て、完了すると次回から出ない状態が記録される / 実測: 登録直後は /projects に着地しウォークスルーは出ない (sawWalk=false)。/t-uc-35 を直接開くと 3 ステップ (ようこそ Atelier へ→ワークスペースを作成→プロジェクトを始める) は進めるが「完了」ボタンは無く (最終: 戻る,次へ(disabled))、再読み込みすると先頭「ようこそ Atelier へ」に戻る。完了状態の記録 (API 呼び出し/localStorage) は無し</t>
+          <t>[再測 R1] 期待: 初回だけ 3 ステップ・完了で次回から出ない / 実測: 登録後 url=/projects 表示=false steps=["最初のワークスペースを作成"] 完了=false ls={} 再表示=false</t>
         </is>
       </c>
     </row>
@@ -3553,12 +3553,12 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J15-03.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J15-03-r1.png</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>期待: 保存後にヘッダーの表示名に反映され、再読み込みしても残る / 実測: PATCH /me 200 で保存は成功し GET /me・再読み込み後の入力値/ヘッダーは「QA jA2 改名太郎」だが、保存直後 (再読み込み前) のヘッダーは旧名「アカウント: QA jA2 1」のまま (G-12: 切替直後に反映されない)。監査ログは未観測</t>
+          <t>[再測 R1] 期待: 保存直後にヘッダー反映・再読み込みでも残る / 実測: PATCH=200 直後反映=false (ヘッダー「Q QA jR1 WS1 Q」) 再読み込み後=false ※本番 web バンドルに GAP-270 の文字列 (atelier:me-changed) が無い = Vercel デプロイが main に追随していない</t>
         </is>
       </c>
     </row>
@@ -3685,12 +3685,12 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J15-05.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J15-05-r1.png</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>期待: 選んだ WS が現在 WS になり、案件一覧がその WS のものに切り替わる / 実測: t-uc-38 で WS2 を選ぶとヘッダーの現在 WS は「QA jA2 WS2」になり localStorage も WS2 で再読み込み後も残る (正) が、/projects の一覧は GET /projects?limit=20 (workspace_id 無し) を叩き「3 件のアクティブプロジェクト」= WS1 の Nebula/Sirius + WS2 の Vega を全部出す = 案件一覧が WS に切り替わらない。加えてヘッダーの現在プロジェクトは WS1 の Nebula のまま (G-13: WS 切替 × 現在案件の組み合わせ)</t>
+          <t>[再測 R1] 期待: 選んだ WS が現在 WS になり案件一覧がその WS に切り替わる (再読み込み後も) / 実測: 現在 WS=WS2 だが一覧は GET ["/projects?limit=20"] で Vega=true Orion=true Sirius=true (WS1 の案件が混在)、現在案件の解除=false (header「Q QA jR1 WS2 / プロジェクト Q」) / 再読み込み後 Vega=true Orion=true Sirius=true ※本番 web バンドルに GAP-271/277 の文字列 (削除済みのプロジェクトはありません / アクティブに戻す) が無い = Vercel デプロイが main (a34f488) に追随していない</t>
         </is>
       </c>
     </row>
@@ -4012,12 +4012,12 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J30-05.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J30-05-r1.png</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>S-B02: 承認待ち 0 (GET /approval-inbox と一致=true), 未解決コメント 1 (一致=true), 最新成果物「要件定義書v2」表示=true, 工程進捗 2/10 表示=false; API task_counts={"triage":2,"ready":0,"in_progress":0,"blocked":0,"awaiting":0,"done":0,"total":2}</t>
+          <t>[再測 R1] 期待: 各カードが実データと一致 / 実測: 工程進捗 1/10 表示=false (画面: 全体進捗率 / 0% / 工程 0/9 完了 / 未承認 INBOX 件数 / 0 / すべて処理済), inbox 一致=true, コメント一致=true, 最新成果物一致=true</t>
         </is>
       </c>
     </row>
@@ -4340,12 +4340,12 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J30-10.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J30-10-r1.png</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>実数表示=true (未完了工程 8 / タスク 2 / 未解決コメント 1 が UI 確認事項と API freeze-check で一致) ; しかし「0 でない間は確定できない」は不成立: UI の確定ボタンは enabled=true、API も残件ありで confirm=true → 200 (捨て案件でフェーズ1 frozen/フェーズ2 active に遷移)</t>
+          <t>[再測 R1] 期待: 実数が出て 0 でない間は確定できない / 実測: 実数表示=true (UI ["・未完了の工程が 9 つあります（提案、見積、契約）","・完了していないタスクが 2 件あります","・未解決のコメントが 3 件あります"] vs API 9/2/3) 確定ボタン enabled=true API freeze=409</t>
         </is>
       </c>
     </row>
@@ -5063,12 +5063,12 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J36-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J36-01-r1.png</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>期待: サイドバーの WS 名に反映 / 実測: PATCH /workspaces 200 で保存され GET も新名だが、保存直後のサイドバー「ワークスペース · QA JA2 WS1 改名」とヘッダー「ワークスペース: QA jA2 WS1 改名」は旧名のまま。再読み込みで初めて「再改名」に変わる (G-12: 直後に反映されない。J15-03 と同型)。※基本情報の保存は POST /account/ai-learning も同時に送る。監査ログ workspace_updated は未観測</t>
+          <t>[再測 R1] 期待: サイドバーに即反映 / 実測: PATCH=200 直後反映=false header「Q QA jR1 WS1 / WS設定 Q」 GET name=QA jR1 WS1 改名</t>
         </is>
       </c>
     </row>
@@ -5392,12 +5392,12 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J36-07.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J36-07-r1.png</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>期待: 30 日案内・一覧から消える・deleted_at 記録・配下データへのアクセス拒否 / 実測: DELETE=204 30日案内=true 一覧から消えた=true GET ws=404 deleted_at=undefined 配下 projects=200/1 詳細=200 employees=200/10。追加: 削除した WS の案件「QA jA2 使い捨て案件」は /projects 一覧 (GET /projects?limit=20) にも出続ける</t>
+          <t>[再測 R1] 期待: 30 日案内・一覧から消える・deleted_at・配下アクセス拒否・監査 / 実測: DELETE=["204 /workspaces/efb95e0c-7021-4509-9121-cca776c5b4d6"] 30日案内=true 一覧残存=false GET ws=404 配下 projects=200/1 詳細=200 employees=200/10 /projects に Vega=true/true</t>
         </is>
       </c>
     </row>
@@ -5523,12 +5523,12 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J37-02.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J37-02-r1.png</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>期待: 名前・口調・「できること」が出て、スキル名や本文は画面と API のどちらにも含まれない (R-T06) / 実測: 名前・口調プリセット・「できること」は出るが、「できること」欄にスキル名 sales-email / proposal / estimate がそのまま列挙され、画面は GET /skills?limit=200 (スキル台帳) も取得。API: GET /ai-employees/{id} は attached_skills にスキル ID 3 件、GET /ai-employees/templates と /templates/{id} は system_prompt 本文 (「あなたは営業・契約部の部長トニーです。…」43 字) を一般利用者に返す = スキル名・本文が漏れる</t>
+          <t>[再測 R1] 期待: 名前・口調・できることが出てスキル名/本文は画面にも API にも無い / 実測: 名前=true 口調=true できること=true 画面スキル語=["sales-email","proposal","estimate"] GET /skills=1 API漏れ=false templates system_prompt=null default_skills=0</t>
         </is>
       </c>
     </row>
@@ -5647,19 +5647,19 @@
           <t>FORBIDDEN_FIELD で拒否され、DB は変わらない</t>
         </is>
       </c>
-      <c r="K79" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K79" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>journeys-A-prod-20260903.txt#J37-04</t>
+          <t>journeys-R1-prod-20260903.txt#J37-04</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>期待: FORBIDDEN_FIELD で拒否・DB 不変 / 実測: 200 {"data":{"id":"2fd8c87c-011a-4419-9d32-6d0be141f908","workspace_id":"3adaebaa-1a52-41c9-8305-b1da3af / 200 {"data":{"id":"2fd8c87c-011a-4419-9d32-6d0be141f908","workspace_id":"3adaebaa-1a52-41c9-8305-b1da3af / 200 / 注入混入=false</t>
+          <t>[再測 R1] system_prompt=422 / attached_skills=422 / 混在 (display_name+system_prompt)=422 で拒否 (detail: "送信内容を確認してください（指示文: この項目は変更できません）。") 。GET 再取得で display_name「トニー」attached_skills も不変・注入文字列の混入なし</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J37-05.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J37-05-r1.png</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>期待: 署名付き URL でアップロードした画像が組織図とチャットに反映され Storage に実体がある / 実測: POST icon-upload-url 200 → 署名付き URL へ PUT 200 → PATCH icon=storage_path 200 → GET icon-url 200 で取得した URL は 200 image/png 79B (Storage に実体あり = G-11 OK)。しかし組織図のノードは頭文字「TO」のまま (img 無し・icon-url の呼び出し無し)、チャット画面も頭文字「ト」= アップロードした画像が画面に反映されない</t>
+          <t>[再測 R1] 期待: 画像が組織図とチャットに反映・Storage に実体 / 実測: upload-url=200 → PUT=200 → PATCH icon=200 → icon-url=200 実体 fetch=200 image/png 70B (Storage に実体あり = G-11 OK) だが、組織図 img=0 (ノード &lt;span aria-label="AI 社員 Tony" role="img" class="inline-flex shrink-0 items-cente, icon-url 呼出 []) チャット img=0 (icon-url 呼出 []) = 画面に画像が反映されない ※本番 web バンドルに GAP-276 の文字列 (ai-employee-icon-url) が無い = Vercel デプロイが main に追随していない</t>
         </is>
       </c>
     </row>
@@ -6048,12 +6048,12 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J38-06.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J38-06-r1.png</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>期待: 一覧からアーカイブ → アクティブ一覧から消えアーカイブ一覧に出る → 戻すと復帰 / 実測: 一覧のカードにアーカイブ/戻す操作が無い (導線: 新規プロジェクト・絞込 すべて/進行中/アーカイブ のみ)。API PATCH status=archived にすると「進行中」絞込からは消え「アーカイブ」絞込に出るが、既定の「すべて」には残り、見出しの件数「3 件のアクティブプロジェクト」も変わらない (GET /projects?limit=20 を 1 回取りクライアント側で絞る)。PATCH status=in_progress で「進行中」に復帰</t>
+          <t>[再測 R1] 期待: 一覧からアーカイブ→アクティブ一覧から消えアーカイブ一覧に出る→戻すと復帰 / 実測: アーカイブ導線=0 すべてに残存=true アーカイブ表示=false 戻す導線=0 復帰=true タブ=["すべて","進行中","アーカイブ","クライアント案件\nヒアリング中\nQA jR1 案件 Sirius (アーカイブ用)\n\n—\n\n工程 1 / 9\n8 分前更新"] ※本番 web バンドルに GAP-277 の文字列 (アクティブに戻す) が無い = Vercel デプロイが main に追随していない</t>
         </is>
       </c>
     </row>
@@ -6106,19 +6106,19 @@
           <t>一覧にマスク表示で出る。応答と DB に平文が無い (暗号化保存)。監査ログ credential_created が記録される</t>
         </is>
       </c>
-      <c r="K86" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K86" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J39-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J39-01-r1.png</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>期待: 一覧にマスク表示・応答/DB に平文無し・監査 credential_created / 実測: 画面の「暗号化して保存」→ POST /projects/{id}/credentials が 500 {"detail":"サーバー側の設定に問題があります。運営にお問い合わせください。"} (API 直接・kind を変えても同じ)。本番に暗号化鍵 (vault key) 等のサーバー設定が無く登録できない (G-11: 外部リソース/秘密の実在)。一覧は 0 件のまま</t>
+          <t>[再測 R1] 「暗号化して保存」→ POST /projects/{id}/credentials 201 (本番の Vault 鍵設定済 = G-11 解消)。一覧にマスク表示 (••••4321) で出て、応答にも GET 一覧にも平文は無い (keys=id,project_id,name,kind,last4,created_by_name,created_at,updated_at)。監査 credential.create は credential 対象で利用者向け API に出ず未観測</t>
         </is>
       </c>
     </row>
@@ -6366,19 +6366,19 @@
           <t>招待が一覧に出て、相手に招待メールが届く (実送信できない環境では送信ログ/キュー投入で代替)。監査ログ invitation_sent が記録される</t>
         </is>
       </c>
-      <c r="K90" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J31-01.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J31-01-r1.png</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>一覧に出る=true (role=member, membership 即時作成)。しかし招待メールは送られない (送信ログ/キュー/API 応答のいずれにも送信の痕跡なし — 実装は登録済みメールを即時 membership 化する方式で、メール送信コードが無い)。監査 workspace_member.invite は admin 専用 API のため未確認</t>
+          <t>[再測 R1] WS 設定の招待フォームで qa-jR1-20260903-2@example.com を招待 → POST /workspaces/{ws}/members 201 → 画面と API の一覧に出る (role=member, 登録済みメールを即時 membership 化)。招待メールは実装 (GAP-281: ResendSender 送信 + 監査 workspace_member.invite_mail) が入ったが、監査ログは WS 対象 (target_type=workspace_membership) で利用者向け API に出ず、応答にも送信結果が無く、受信箱も無い = 送信の痕跡を観測できない / 解除条件: 運営の /admin/audit-logs で workspace_member.invite_mail (dry_run / email_id) を照会、または受信箱</t>
         </is>
       </c>
     </row>
@@ -6693,19 +6693,19 @@
           <t>編集操作は 403 で拒否され、閲覧は引き続きできる状態である</t>
         </is>
       </c>
-      <c r="K95" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J31-06.png</t>
+          <t>journeys-R1-prod-20260903.txt#J31-06</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>ロール変更直後・同じトークンで: 案件名変更=403, タスク作成=500 (403 期待), 閲覧 GET project=200 tasks=200; 案件名不変=true</t>
+          <t>[再測 R1] 閲覧者: 案件名変更 403「このプロジェクトを変更する権限がありません。」/ タスク作成 403「この操作を行う権限がありません。」(GAP-282: RLS 拒否が 500 でなく 403)。閲覧 GET project 200 / tasks 200 は引き続き可。案件名は不変</t>
         </is>
       </c>
     </row>
@@ -6765,12 +6765,12 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J31-07.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J31-07-r1.png</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>閲覧者: シークレット追加=500「サーバー側の設定に問題があります」(403 期待), reveal=404 (対象なし)。根本原因: owner による事前登録 (J39-01 相当) も 500 → 本番にシークレット暗号鍵 (Fernet) が未設定 (G-11)。認可 (403) より先に設定エラーが返るため、閲覧者判定も未達。値漏れ=false, 一覧 GET=200 (0 件)。監査の拒否記録は admin 専用 API のため未確認</t>
+          <t>[再測 R1] 期待: 追加・reveal とも 403 で値は漏れない・監査に拒否 / 実測: 追加は 403「シークレットを追加する権限がありません。」(GAP-278 ② OK) だが **reveal は 403 でなく 200 で平文を返す** (role=viewer の閲覧者が本人パスワードで再認証すると owner が登録したシークレット値がそのまま取れる = 値が漏れる。R-T06 級の権限漏れ)。画面 (S-B04) にも閲覧者に「表示」ボタンが出る。監査の拒否記録は利用者向け API に出ず未観測。再現: viewer の JWT で POST /projects/{pid}/credentials/{cid}/reveal {"password":"&lt;redacted&gt;"} → 200 {"value":"&lt;redacted&gt;"}</t>
         </is>
       </c>
     </row>
@@ -6831,12 +6831,12 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J31-08.png</t>
+          <t>journeys-R1-prod-20260903.txt#J31-08</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>招待リンク・expires_at を持つ招待エンティティが実装に存在しない (POST /workspaces/{id}/members は登録済みメールを即時 membership 化し、招待一覧/期限/リンクの API・UI が無い)。「7 日で期限切れ」の仕様を満たす対象が無いため期待未達</t>
+          <t>[再測 R1] 期待: 期限切れ (7 日) の招待リンクが拒否される / 実測: WS 招待にリンク・expires_at を持つ招待エンティティが依然として無い (未登録メールは 422「このメールアドレスのアカウントは登録されていません。」で招待自体が作れず、メンバー行の keys=workspace_id,user_id,email,display_name,role,joined_at に期限は無い。GET /workspaces/{id}/invitations は 404)。GAP-281 で「招待リンク / 有効期限は仕様未確定のため別途 (T-A-30)」と保留のまま = 期限切れの対象が存在しない</t>
         </is>
       </c>
     </row>
@@ -7085,19 +7085,19 @@
           <t>LAST_OWNER エラーで拒否され、メンバー一覧は変わらない (DB の membership も残る)</t>
         </is>
       </c>
-      <c r="K101" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K101" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J36-06.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J36-06-r1.png</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>期待: LAST_OWNER エラーで拒否され一覧不変 / 実測: 画面のメンバー一覧には自分 (唯一の owner) の削除ボタンが無い。API 直接 DELETE /workspaces/{ws}/members/{自分} は 204 (2 回実行とも) を返すが membership は残る (1 名 owner のまま) = エラーではなく「成功したふりの no-op」。期待の LAST_OWNER エラーが返らない</t>
+          <t>[再測 R1] API DELETE /workspaces/{ws}/members/{自分} → 409「最後の owner は外せません。先に別のメンバーを owner にしてください。」で拒否、メンバー一覧は 1 名 (owner) のまま。UI のメンバー一覧には唯一の owner の削除ボタンが 0 個 (出ない)</t>
         </is>
       </c>
     </row>
@@ -11153,12 +11153,12 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J34-06.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J34-06-r1.png</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>.exe: UI の input は accept="audio/*,video/*,.txt,.md,.docx,text/plain" で選択を絞るだけで、選択できてしまえば (D&amp;D/強制選択) そのまま送信され、日本語エラーは出ず一覧に「setup.exe / 102 B / 解析中」で増えた (後の一覧再確認で表示を確認)。API も upload-url=200 / POST /meetings (mime application/x-msdownload)=201 で拒否しない → 期待 (日本語エラーで拒否・一覧に増えない) 未達</t>
+          <t>[再測 R1] 期待: 日本語エラーで拒否・一覧に増えない / 実測: 画面文言=「Atelier API POST /meetings/upload-url -&gt; 422 | エラー | 解析に失敗したため、結果を表示できません。」 一覧 exe=false API upload-url=422 POST=422</t>
         </is>
       </c>
     </row>
@@ -11348,12 +11348,12 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>evidence/journeys-B-prod-20260903.txt</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J35-01-r1.png</t>
         </is>
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>POST /knowledge 201 → GET /knowledge (workspace) 一覧に出る=True。しかし埋め込みは生成されない: GET /embedding-status provider=none state=unavailable indexed/total=0/1 semantic_enabled=false (本番に埋め込みプロバイダが未設定 = G-11)。監査ログ knowledge.create は利用者向け API に露出せず未確認</t>
+          <t>[再測 R1] 期待: 一覧に出て埋め込みが生成される (embedding-status に反映)・監査 / 実測: POST=201 一覧 (API/画面)=true/true だが埋め込みは生成されない: GET /embedding-status provider=none state=unavailable semantic_enabled=false reason=「意味検索の部品 (fastembed) がこのサーバーに入っていません (キーワード一致のみ)」= 本番に埋め込みプロバイダ (fastembed) が依然未導入 (G-11、GAP-285 ①は経営判断のまま)。監査 knowledge.create は利用者向け API に出ず未観測</t>
         </is>
       </c>
     </row>
@@ -11677,12 +11677,12 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J35-07.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J35-07-r1.png</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>状態カードに何で動くか/費用=表示あり (意味検索は使えません（キーワード一致のみ） / 費用なし /  / 意味検索の部品 (fastembed) がこのサーバーに入っていません (キーワード一致のみ) /  / 埋め込); 「再試行する」押下 → 処理中に遷移=true, 完了 (ready)=false: サーバーに fastembed が無く provider=none/unavailable のまま (G-11: 本番に意味検索の部品が未導入)。検索はキーワード一致で 0 件</t>
+          <t>[再測 R1] 期待: 何で動いていて誰の費用かが出て、準備を押すと処理中→完了後に検索で引ける / 実測: 状態カードに何で動くか・費用=true (「意味検索は使えません（キーワード一致のみ） / 費用なし / 意味検索の部品 (fastembed) がこのサーバーに入っていません (キーワード一致のみ) / 埋め込み済み 0 」)。「再試行する」押下 → POST /embedding-status/prepare は 503 で理由を返し (GAP-285 ②: 「準備を開始しました」と偽らない=true)、状態は provider=none state=unavailable のまま = 本番に埋め込みプロバイダ (fastembed) が未導入で処理中→完了に遷移しない (G-11、GAP-285 ①は経営判断のまま)</t>
         </is>
       </c>
     </row>
@@ -13306,19 +13306,19 @@
           <t>トークンがローテーションされ新リンクがメールで届く (実送信できない環境では送信ログ/キュー投入で代替)。旧リンクは無効になる</t>
         </is>
       </c>
-      <c r="K196" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K196" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/journeys-E-prod-20260903.txt</t>
+          <t>journeys-R1-prod-20260903.txt#J20-05</t>
         </is>
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>resend が 409: {"detail": "この招待はすでに使われたか、取り消されています。"}</t>
+          <t>[再測 R1] 使用済み (used_at 有) の招待で再送 200 → token がローテーション (旧≠新)。旧リンク preview 401 / signin 401 で無効、新リンク preview 200 / signin 200。メール送信の痕跡は利用者向け API に露出せず未観測 (受信箱なし)。付記 (G-12): 再送前に発行済みのクライアント券は GET /client/projects → 200</t>
         </is>
       </c>
     </row>
@@ -13696,19 +13696,19 @@
           <t>招待者に更新のメールが届く (実送信できない環境では送信ログ/キュー投入で代替)。監査ログ client_notified_of_update が記録される</t>
         </is>
       </c>
-      <c r="K202" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K202" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/journeys-E-prod-20260903.txt</t>
+          <t>journeys-R1-prod-20260903.txt#J21-05</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>期待: 成果物の新版で招待者に更新メール + 監査ログ client_notified_of_update / 実測: 新版 (要件定義 v3) 作成は 200 だが、更新通知メールを送る実装が API に存在しない (ResendSender の呼出箇所に成果物更新が無い)。観測できる送信痕跡も無し。T-F-17 未実装扱い</t>
+          <t>[再測 R1] 新版 (要件定義 v2) の作成は 200。送信の実装 (services/outputs/client_notify.py) は入ったが、監査ログ output.client_notified_of_update は target=workflow_output で書かれ、利用者が読める API (dashboard recent_activities は project/task/comment 対象のみ) に出ない。import 応答 (keys=file_name,type,title,stage,version,target_id,error) にも送信結果が無く、受信箱も無い / 解除条件: 運営の /admin/audit-logs で action=output.client_notified_of_update を照会するか、dashboard の監査に成果物対象を含める</t>
         </is>
       </c>
     </row>
@@ -14023,19 +14023,19 @@
           <t>コメントが自分の画面の一覧に出る。担当者に通知メールが届く (実送信できない環境では送信ログ/キュー投入で代替)。監査ログ comment_created が記録される</t>
         </is>
       </c>
-      <c r="K207" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K207" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/journeys-E-prod-20260903.txt</t>
+          <t>journeys-R1-prod-20260903.txt#J23-01</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>期待: 一覧に出る + 担当者に通知メール + 監査ログ comment_created / 実測: POST /client/projects/PE1/comments 201、自分の一覧に出る (is_client_author=true) は OK。しかし担当者への通知メールを送る実装が API に無い (services/client_signin・comments に Resend/notify 呼出なし, grep 0 件) → 送信痕跡も無し。監査ログは admin 専用で未確認</t>
+          <t>[再測 R1] POST /client/projects/{id}/comments 201 → 自分の一覧に出る (is_client_author=true)。担当者 (WS owner) への通知は監査ログ client.comment.staff_notified が owner のダッシュボード recent_activities に記録された (client.comment.staff_notified,client.comment.create) = 送信 (dry-run 含む) の痕跡。受信箱は無いので実受信は未確認</t>
         </is>
       </c>
     </row>
@@ -14162,12 +14162,12 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/journeys-E-prod-20260903.txt</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J23-03-r1.png</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>期待: 自分のコメントは編集・削除できる / 実測: クライアント用の編集・削除 endpoint が無い (PATCH/DELETE /client/projects/{id}/comments/{id} → 404 Not Found、社内 PATCH/DELETE /comments/{id} は client 券で 401)。S-L03 にも編集/削除ボタン 0 個。他人 (社内メモ) の編集は 401 で拒否され content 不変 (こちらは OK)</t>
+          <t>[再測 R1] 期待: 自分のものは編集・削除が反映、他人のものは拒否 / 実測: API 直では PATCH/DELETE /client/projects/{pid}/comments/{cid} が 自分=200/204 (反映 true/true)・他人=404/404 (不変 true) で期待どおり (GAP-267 API 稼働、監査 client.comment.update/delete あり) だが、画面 S-L03 に「修正」0 個・「取り消す」0 個 = クライアントは画面から編集・削除できない ※本番 web バンドルが main に追随しておらず GAP-267 web 側が未反映</t>
         </is>
       </c>
     </row>
@@ -14557,12 +14557,12 @@
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J38-03.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J38-03-r1.png</t>
         </is>
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>期待: 30 日カウントダウンつきで一覧から消え (deleted_at 記録)、クライアント招待が無効化、監査 project_deleted / 実測: 設定の危険な操作から削除 (DELETE 204) でアクティブ一覧から消え include_deleted で deleted_at=2026-09-03T05:23:54Z。削除後の招待 token は POST /client/auth/preview 401 (削除前は 200) で無効化 (ただし GET 招待の revoked_at は null のまま = 暗黙無効)。不足: 削除後に「残り N 日」のカウントダウンや削除済み一覧が画面のどこにも無い (30 日の文言は削除前の確認ダイアログのみ)。監査 project.delete は削除後ダッシュボードが 404 で観測不可</t>
+          <t>[再測 R1] 期待: 30 日カウントダウンつきで一覧から消える (deleted_at)・クライアント招待無効化・監査 project_deleted / 実測: DELETE=204 アクティブ一覧から消えた=true deleted_at=2026-09-03T07:46:48.129161Z (API は記録)・招待 preview 200→401 / 発行済み券 GET 401 (無効化 OK) だが、画面に「削除済み」タブ/カウントダウンが無い (タブ=["すべて","進行中","アーカイブ"], 30 日の文言は削除前の確認「危険な操作 / プロジェクト削除は 30 日後にハード削除されます。30 日以内であればキャンセル可能。 / プロジェク」のみ) ※本番 web バンドルに GAP-277 の文字列が無い = Vercel デプロイが main に追随していない</t>
         </is>
       </c>
     </row>
@@ -14622,12 +14622,12 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J38-04.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J38-04-r1.png</t>
         </is>
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t>期待: 削除済み一覧から復元し、元の状態に戻り成果物・タスク・コメントが残る / 実測: 画面 (/projects) に削除済み一覧も復元ボタンも無く、利用者は画面から復元できない。API POST /projects/{id}/restore は 200 で deleted_at が消えて一覧に戻り、タスク「QA jA2 タスク Nebula-TASK-1」とコメントは残っている (データ面は正)</t>
+          <t>[再測 R1] 期待: 削除済み一覧から復元し元の状態に戻る / 実測: 画面に削除済み一覧・復元導線が無い (UI 復元=null)。API POST /projects/{id}/restore 200 で deleted_at が消え一覧に戻り、タスク 2 件・成果物 3 件・コメント 4 件は残る (データ面は正)。J38-03 の監査 project.delete が dashboard に出る=true ※本番 web バンドルに GAP-277 の文字列が無い = Vercel デプロイが main に追随していない</t>
         </is>
       </c>
     </row>
@@ -18804,19 +18804,19 @@
           <t>入れない状態で、理由が日本語で分かる。復元の導線だけが出る</t>
         </is>
       </c>
-      <c r="K280" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K280" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/journeys-E-prod-20260903.txt</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J52-03-r1.png</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>期待: 入れず理由が日本語で分かる・復元導線だけが出る / 実測: 退会後 signin は 401『メールアドレスまたはパスワードが違います。』(API/UI とも) で『退会中』という理由が分からない (パスワード誤りと区別不能)。復元リンクはサインイン画面に常時ある汎用リンクで、退会中に限って出るものではない。※存在秘匿の設計判断ならその旨を正本に明記して期待を改訂する</t>
+          <t>[再測 R1] 退会申込後に正しいパスワードで UI サインイン → API 403、画面に「このアカウントは退会手続き中です。サインイン画面の「退会済みアカウントの復元」から 30 日以内であれば復元できます。」と日本語で理由が出て入れない。復元の導線 ["退会済みアカウントの復元"] が出る。対照: 誤パスワードは従来どおり 401「メールアドレスまたはパスワードが違います。」(存在を漏らさない)</t>
         </is>
       </c>
     </row>
@@ -19073,12 +19073,12 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J30-15.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J30-15-r1.png</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>共有リンク発行 → 公開 GET /share/{token} (認証なし)=200 で最終版が見える (クライアント側 J21 の代替); 納品工程 confirm なし 403 / confirm あり 200 → flow delivery=done。しかし案件の状態は納品済みにならない: GET /projects/{id}.status=draft, 一覧 status=draft, dashboard status=draft current_phase=hearing; 画面 (一覧/ダッシュボード) に納品済み表記=false</t>
+          <t>[再測 R1] 期待: 納品工程 done・案件が納品済みとして一覧とダッシュボードに反映・クライアントに最終版 / 実測: delivery complete=200 flow delivery=done API current_phase=delivery/delivery/delivery status=draft (API は納品済み=true) / 画面: 一覧カード「のアクティブプロジェクト / 新規プロジェクト / プロジェクトを検索 / すべて / 進行中 / アーカイブ / クライアント案件 / 納品済 / QA jR」 ダッシュボード「プロジェクトダッシュボード / QA jR1 案件 Orion · クライアント案件 · 第 1 段階 ヒアリング中 / 全体進捗率 / 0% / 工程 0/9」 進捗「全体進捗率 / 0% / 工程 0/9 完了 / 未承認 INBOX 件数 / 0 / すべて処理済」 (画面は納品済み=false) / クライアント delivery=true ※本番 web バンドルが main に追随していない (GAP-279 の web 側「進捗カードも flow を優先」未反映の可能性)</t>
         </is>
       </c>
     </row>
@@ -19132,19 +19132,19 @@
           <t>owner 側のボードとダッシュボードに完了とコメントが反映される。監査ログ task_status_changed / comment_created が記録される</t>
         </is>
       </c>
-      <c r="K285" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K285" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L285" t="inlineStr">
         <is>
-          <t>evidence/shots/journeys/J31-12.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J31-12-r1.png</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>タスク完了=200/done, コメント=201; owner ダッシュボード done=1 未解決コメント=2 (画面反映=true); 監査 recent_activities=["project.flow.thread","task.create","task.create","project.flow.complete"] → task 系=false, comment 系=false (comment_created 相当は project/task 対象の audit にしか出ないため未確認)</t>
+          <t>[再測 R1] メンバーがタスク A を done (PATCH 200) にしコメント (201) → owner のダッシュボード API で done 0→1・未解決コメント 3→4、画面のダッシュボードも「未解決コメント / 4 / 確定 0 · 未確認 0 件 / 工程の流れ」。監査 recent_activities に task.update / comment.create (メンバーの行為) が出る (comment.create,task.update,task.create)</t>
         </is>
       </c>
     </row>
@@ -19205,12 +19205,12 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/journeys-E-prod-20260903.txt</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J23-05-r1.png</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>返信は自分のコメントの下に表示 (OK)。しかし納品成果物は S-L03 に『納品書 2026/09/03 · v1 · HTML』の行として出るだけで、開く導線 (リンク/ボタン) が無く、client 用の content/content-url API も openapi に無い → 『納品された最終版の成果物が閲覧できる状態』を満たさない (行をクリックしても遷移・API 呼出なし)</t>
+          <t>[再測 R1] 期待: 返信が自分のコメントの下・納品最終版が閲覧できる / 実測: 返信の表示=false、納品成果物の行=true だが「開く」導線=0 個 (content-url 呼出 []) = 画面からは開けない。API 側は GET /client/projects/{pid}/outputs/{oid}/content-url → 200 で実体 200 本文に納品物あり (GAP-268 の API は稼働) ※本番 web バンドルが main に追随しておらず S-L03 の「開く」(GAP-268 web 側) が未反映</t>
         </is>
       </c>
     </row>
@@ -21404,11 +21404,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>39%</t>
         </is>
       </c>
     </row>
@@ -21419,11 +21419,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>11%</t>
         </is>
       </c>
     </row>
@@ -21434,11 +21434,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>49%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(正本): GAP-319/320 起票、SG01-906 / SC02-902 追加、通し R3 再測 (18 行: PASS 14 / FAIL 3 / BLOCKED 1) を集約
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/apps/web/.qa/e2e-journey/journey-20260903.xlsx
+++ b/apps/web/.qa/e2e-journey/journey-20260903.xlsx
@@ -2294,19 +2294,19 @@
           <t>日本語のエラーで拒否され、ワークスペースは増えない</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J10-07-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J10-07-r3.png</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 日本語エラーで拒否・WS 増えない / 実測: errors=[] POST=未送信 disabled=true WS 件数=0</t>
+          <t>[再測 R3] 名前を空のまま作成すると画面に日本語のエラー ["ワークスペース名を入力してください。"] が出て拒否される (GAP-263)。POST /workspaces は 送信されず、GET /workspaces も 0 件のままでワークスペースは増えない</t>
         </is>
       </c>
     </row>
@@ -3481,19 +3481,19 @@
           <t>初回だけ 3 ステップのウォークスルーが出る。完了すると次回から出ない状態が記録される</t>
         </is>
       </c>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J15-01-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J15-01-r3.png</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 初回だけ 3 ステップ・完了で次回から出ない / 実測: 登録後 url=/projects 表示=false steps=["最初のワークスペースを作成"] 完了=false ls={} 再表示=false</t>
+          <t>[再測 R3] 新規登録の直後に /t-uc-35 のウォークスルーが出て、3 ステップ ["ようこそ Atelier へ","ワークスペースを作成","プロジェクトを始める"] を「完了」まで進めると /projects へ戻る。完了状態が localStorage atelier_walkthrough_done=1 に記録され、以後 /t-uc-35 を直接開いても /t-uc-35 へ抜け、/projects を再読み込みしてもウォークスルーは出ない (GAP-262)</t>
         </is>
       </c>
     </row>
@@ -3546,19 +3546,19 @@
           <t>保存後にヘッダーの表示名に反映され、再読み込みしても残る。監査ログに記録される</t>
         </is>
       </c>
-      <c r="K47" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J15-03-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J15-03-r3.png</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 保存直後にヘッダー反映・再読み込みでも残る / 実測: PATCH=200 直後反映=false (ヘッダー「Q QA jR1 WS1 Q」) 再読み込み後=false ※本番 web バンドルに GAP-270 の文字列 (atelier:me-changed) が無い = Vercel デプロイが main に追随していない</t>
+          <t>[再測 R3] T-UC-37 で表示名を保存 (PATCH /me 200) → 再読み込みなしでヘッダーのアカウント表示が「アカウント: QA jR3 改名花子」に変わり (GAP-270 の atelier:me-changed でシェルが /me を読み直す)、メニューの氏名行も新名。再読み込み後も「アカウント: QA jR3 改名花子」・GET /me も同じ。監査ログは利用者向け API に露出せず未観測</t>
         </is>
       </c>
     </row>
@@ -3678,19 +3678,19 @@
           <t>選んだワークスペースが現在のワークスペースとして反映され、案件一覧がそのワークスペースのものに切り替わる。再読み込み後も残る</t>
         </is>
       </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J15-05-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J15-05-r3.png</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 選んだ WS が現在 WS になり案件一覧がその WS に切り替わる (再読み込み後も) / 実測: 現在 WS=WS2 だが一覧は GET ["/projects?limit=20"] で Vega=true Orion=true Sirius=true (WS1 の案件が混在)、現在案件の解除=false (header「Q QA jR1 WS2 / プロジェクト Q」) / 再読み込み後 Vega=true Orion=true Sirius=true ※本番 web バンドルに GAP-271/277 の文字列 (削除済みのプロジェクトはありません / アクティブに戻す) が無い = Vercel デプロイが main (a34f488) に追随していない</t>
+          <t>[再測 R3] t-uc-38 の切替で WS2 を選ぶと現在 WS が WS2 になり (ヘッダーも WS2)、/projects は GET /projects?limit=20&amp;include_deleted=true&amp;workspace_id=a6e16ef で WS2 の Vega だけ (WS1 の Orion / Sirius は出ない = GAP-271)。現在案件も旧 WS の Orion から解除。再読み込み後も WS2・Vega のまま</t>
         </is>
       </c>
     </row>
@@ -4005,19 +4005,19 @@
           <t>各カードが実データと一致して反映される。承認待ちの件数は GET /approval-inbox の件数と同じ</t>
         </is>
       </c>
-      <c r="K54" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J30-05-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J30-05-r3.png</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 各カードが実データと一致 / 実測: 工程進捗 1/10 表示=false (画面: 全体進捗率 / 0% / 工程 0/9 完了 / 未承認 INBOX 件数 / 0 / すべて処理済), inbox 一致=true, コメント一致=true, 最新成果物一致=true</t>
+          <t>[再測 R3] S-B02: 工程進捗「工程 1/10」(flow の done 数と一致・GAP-279)、承認待ち 0 (GET /approval-inbox と一致)、未解決コメント 3 (unresolved-count と一致)、最新成果物「要件定義書 QA-R3」が実データと一致。project.current_phase=hearing</t>
         </is>
       </c>
     </row>
@@ -4333,19 +4333,19 @@
           <t>未完了工程・タスク・未解決コメントの実数が出る。0 でない間は確定できない状態である</t>
         </is>
       </c>
-      <c r="K59" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J30-10-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J30-10-r3.png</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 実数が出て 0 でない間は確定できない / 実測: 実数表示=true (UI ["・未完了の工程が 9 つあります（提案、見積、契約）","・完了していないタスクが 2 件あります","・未解決のコメントが 3 件あります"] vs API 9/2/3) 確定ボタン enabled=true API freeze=409</t>
+          <t>[再測 R3] 確定前チェックに未完了工程 9 / タスク 2 / 未解決コメント 3 の実数 (API freeze-check と一致) が出て、確定ボタンは無効 (残件を承知するチェックまで押せない・GAP-280)。API も残件ありの confirm=true は 409「残っている作業があるため確定できません（未完了の工程が 9 つあります（提案、見積、契約） / 完了していないタスクが 2 件あります / 」で確定できない (フェーズは active のまま)</t>
         </is>
       </c>
     </row>
@@ -5056,19 +5056,19 @@
           <t>サイドバーのワークスペース名に反映され、監査ログ workspace_updated が記録される</t>
         </is>
       </c>
-      <c r="K70" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J36-01-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J36-01-r3.png</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: サイドバーに即反映 / 実測: PATCH=200 直後反映=false header「Q QA jR1 WS1 / WS設定 Q」 GET name=QA jR1 WS1 改名</t>
+          <t>[再測 R3] PATCH /workspaces 200 → 保存直後 (再読み込みなし) にサイドバー/ヘッダーが「QA jR3 WS1 改名」に変わり (GAP-270)、GET も新名。監査ログ workspace.update は WS 対象で利用者向け API (dashboard) に出ず未観測</t>
         </is>
       </c>
     </row>
@@ -5385,19 +5385,19 @@
           <t>30 日保持の案内が出て一覧から消える。DB に deleted_at が記録され、そのワークスペースのデータへのアクセスは拒否される。監査ログ workspace_deleted が記録される</t>
         </is>
       </c>
-      <c r="K75" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J36-07-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J36-07-r3.png</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 30 日案内・一覧から消える・deleted_at・配下アクセス拒否・監査 / 実測: DELETE=["204 /workspaces/efb95e0c-7021-4509-9121-cca776c5b4d6"] 30日案内=true 一覧残存=false GET ws=404 配下 projects=200/1 詳細=200 employees=200/10 /projects に Vega=true/true</t>
+          <t>[再測 R3] WS 設定の退会タブに「ワークスペースの削除 / Danger Zone / ワークスペース削除は 30 日後にハード削除されます。30 日以内であればキャンセル可能。 / ワークスペースを削除 / アカ」と 30 日保持の案内が出た上で削除 (DELETE 204) → GET /workspaces から消え、GET /workspaces/{id} は 404。配下へのアクセスも拒否され (GET /projects?workspace_id → 200 0 件 / GET /projects/{Vega} → 404 / GET /ai-employees?workspace_id → 200 0 名)、/projects?limit=20 にも画面の一覧にも Vega は出ない = GAP-273 の RLS helper が migration 改名 (t-d-99zt) で本番に効いている (R1 では配下が 200 で読めていた)。deleted_at は 削除後は 404 で API から直接読めない (削除の事実は 404 と配下拒否で確認)。監査 workspace.delete は WS 対象で利用者向け API に出ず未観測</t>
         </is>
       </c>
     </row>
@@ -5523,12 +5523,12 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J37-02-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J37-02-r3.png</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 名前・口調・できることが出てスキル名/本文は画面にも API にも無い / 実測: 名前=true 口調=true できること=true 画面スキル語=["sales-email","proposal","estimate"] GET /skills=1 API漏れ=false templates system_prompt=null default_skills=0</t>
+          <t>[再測 R3] 期待: 名前・口調・できること が出て、スキル名や本文は画面と API 応答のどちらにも含まれない / 実測: 画面は改善 (名前=true 口調=true できること=true、チップは説明文「成 / 提案書作成 / 見積作成 / 担当範囲 / 役職 / 部長 / 所属 / 営業・契約部 / レポート対象 / ジャービス / 直属の部下 / メンバー 」でスキル名の露出=0 個・GAP-274 の web 側は反映済) だが、**この画面は今も GET /skills を 1 回呼び、その応答 (200, 23 件, keys=id,name,version,description,is_active) に内部スキル名が入っている** (この社員の attached_skills 3 件 = ["sales-email","proposal","estimate"])。= API 応答にスキル名が含まれる状態のまま (R-T06)。templates 側は system_prompt=null / default_skills=0 で秘匿済み</t>
         </is>
       </c>
     </row>
@@ -5713,19 +5713,19 @@
           <t>署名付き URL でアップロードした画像が組織図とチャットに反映される。Storage に実体が存在する (G-11)</t>
         </is>
       </c>
-      <c r="K80" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J37-05-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J37-05-r3.png</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 画像が組織図とチャットに反映・Storage に実体 / 実測: upload-url=200 → PUT=200 → PATCH icon=200 → icon-url=200 実体 fetch=200 image/png 70B (Storage に実体あり = G-11 OK) だが、組織図 img=0 (ノード &lt;span aria-label="AI 社員 Tony" role="img" class="inline-flex shrink-0 items-cente, icon-url 呼出 []) チャット img=0 (icon-url 呼出 []) = 画面に画像が反映されない ※本番 web バンドルに GAP-276 の文字列 (ai-employee-icon-url) が無い = Vercel デプロイが main に追随していない</t>
+          <t>[再測 R3] (ui2 の FAIL 行を上書き) 署名 URL 発行 200 → PUT 200 → PATCH icon 200 → GET icon-url 200 → 実体 200 image/png 70B (Storage に実在 = G-11 OK)。組織図 (S-C01) は署名 URL の img 1 枚で画像に差し替わる (icon-url 呼出 200 = GAP-276 の web 側は本番に反映済)。チャット (S-E01) も icon-url を 200 で引き iconSrc を ChatPanel へ渡しているが、**アップロード画像が描画されるのは assistant ロールのメッセージ行だけ**で、AI 応答が 1 件も無いスレッドでは img が 0 のまま = 画面上で確認できない。GET /bridge/status は running/queued 0・active_worker_pids [] で AI を動かせない / 解除条件: Bridge (場所=mac) で AI 応答を 1 件出したスレッドを開き、その行のアイコンが画像かを見る</t>
         </is>
       </c>
     </row>
@@ -6041,19 +6041,19 @@
           <t>アクティブ一覧から消えアーカイブ一覧に出る。戻すとアクティブ一覧に反映される</t>
         </is>
       </c>
-      <c r="K85" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J38-06-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J38-06-r3.png</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 一覧からアーカイブ→アクティブ一覧から消えアーカイブ一覧に出る→戻すと復帰 / 実測: アーカイブ導線=0 すべてに残存=true アーカイブ表示=false 戻す導線=0 復帰=true タブ=["すべて","進行中","アーカイブ","クライアント案件\nヒアリング中\nQA jR1 案件 Sirius (アーカイブ用)\n\n—\n\n工程 1 / 9\n8 分前更新"] ※本番 web バンドルに GAP-277 の文字列 (アクティブに戻す) が無い = Vercel デプロイが main に追随していない</t>
+          <t>[再測 R3] 一覧カードの「アーカイブ」(PATCH 200) で Sirius がアクティブ (すべて) から消え「アーカイブ」タブに出る。「アクティブに戻す」(PATCH 200) で「すべて」に復帰 (API status=in_progress) — GAP-277 の web 側が反映済</t>
         </is>
       </c>
     </row>
@@ -6765,12 +6765,12 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J31-07-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J31-07-r3.png</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 追加・reveal とも 403 で値は漏れない・監査に拒否 / 実測: 追加は 403「シークレットを追加する権限がありません。」(GAP-278 ② OK) だが **reveal は 403 でなく 200 で平文を返す** (role=viewer の閲覧者が本人パスワードで再認証すると owner が登録したシークレット値がそのまま取れる = 値が漏れる。R-T06 級の権限漏れ)。画面 (S-B04) にも閲覧者に「表示」ボタンが出る。監査の拒否記録は利用者向け API に出ず未観測。再現: viewer の JWT で POST /projects/{pid}/credentials/{cid}/reveal {"password":"&lt;redacted&gt;"} → 200 {"value":"&lt;redacted&gt;"}</t>
+          <t>[再測 R3] (ui3 の行を詳細化) 期待: 追加と表示のどちらも 403 で拒否され値は漏れない・監査に拒否が記録される。実測: **API は両方 403 に直った** — 閲覧者 (role=viewer) の POST /projects/{p}/credentials → 403「シークレットを追加する権限がありません。」、POST /projects/{p}/credentials/{c}/reveal は本人パスワードつきでも無しでも 403「シークレットの値を表示する権限がありません。」で平文は返らない (GAP-313 修正が本番で効いている。R1 では 200 で平文が返っていた)。一覧 GET は 200 でマスク (last4 のみ)、owner 側の一覧も 1 件のままで閲覧者の追加は入らない。**しかし画面 S-B04 は閲覧者にも「表示」ボタン 1 個と追加フォーム (#cred-name / #cred-kind / #cred-value / 「暗号化して保存」) と「QA jR3 顧客 API キー を削除」を出したまま** = 押せば 403 になるだけの操作を見せている (GAP-313 の「画面側の『表示』非表示」は未実装。app/projects/s_b04/_components/CredentialList.tsx / CredentialForm.tsx にロール判定が無い)。監査ログの拒否記録は credential 対象で利用者向け API に出ず未観測。再現: viewer の JWT で /projects/vault?project={pid} を開く → 「表示」ボタンと追加フォームが出る</t>
         </is>
       </c>
     </row>
@@ -11146,19 +11146,19 @@
           <t>日本語のエラーで拒否され、一覧に増えない</t>
         </is>
       </c>
-      <c r="K163" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K163" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J34-06-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J34-06-r3.png</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 日本語エラーで拒否・一覧に増えない / 実測: 画面文言=「Atelier API POST /meetings/upload-url -&gt; 422 | エラー | 解析に失敗したため、結果を表示できません。」 一覧 exe=false API upload-url=422 POST=422</t>
+          <t>[再測 R3] .exe を選んで送ると画面に「対応していない形式です (.exe)。音声・動画・テキスト (.txt / .md)・Word (.docx) のみ登録できます。 | エラー | 解析に失敗したため、結果を表示できません。」と日本語だけで拒否され (GAP-314: 内部の英語メソッド/パス/status は出ない)、一覧に増えない (0 件のまま)。API 直でも upload-url / POST /meetings とも 422「対応していない形式です (.exe)。音声・動画・テキスト (.txt / .md)・Word (.docx) のみ登録」</t>
         </is>
       </c>
     </row>
@@ -14155,19 +14155,19 @@
           <t>自分のものは編集・削除が反映される。他人のものは拒否される</t>
         </is>
       </c>
-      <c r="K209" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K209" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J23-03-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J23-03-r3.png</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 自分のものは編集・削除が反映、他人のものは拒否 / 実測: API 直では PATCH/DELETE /client/projects/{pid}/comments/{cid} が 自分=200/204 (反映 true/true)・他人=404/404 (不変 true) で期待どおり (GAP-267 API 稼働、監査 client.comment.update/delete あり) だが、画面 S-L03 に「修正」0 個・「取り消す」0 個 = クライアントは画面から編集・削除できない ※本番 web バンドルが main に追随しておらず GAP-267 web 側が未反映</t>
+          <t>[再測 R3] S-L03 の自分のコメントに「修正」2 個・「取り消す」2 個が出る (GAP-267 の web 側が本番に反映済)。画面から修正 → PATCH 200 で表示も API 再取得も修正後の本文に、画面から取り消す → DELETE 204 で画面と API 一覧から消える。社内 (他人) の返信には操作導線が出ず、API 直でも PATCH 404 / DELETE 404 で拒否され本文は不変。監査 client.comment.delete,client.comment.update</t>
         </is>
       </c>
     </row>
@@ -14550,19 +14550,19 @@
           <t>30 日カウントダウンつきで一覧から消える (deleted_at が記録)。その案件のクライアント招待は無効化され、監査ログ project_deleted が記録される</t>
         </is>
       </c>
-      <c r="K215" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K215" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J38-03-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J38-03-r3.png</t>
         </is>
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 30 日カウントダウンつきで一覧から消える (deleted_at)・クライアント招待無効化・監査 project_deleted / 実測: DELETE=204 アクティブ一覧から消えた=true deleted_at=2026-09-03T07:46:48.129161Z (API は記録)・招待 preview 200→401 / 発行済み券 GET 401 (無効化 OK) だが、画面に「削除済み」タブ/カウントダウンが無い (タブ=["すべて","進行中","アーカイブ"], 30 日の文言は削除前の確認「危険な操作 / プロジェクト削除は 30 日後にハード削除されます。30 日以内であればキャンセル可能。 / プロジェク」のみ) ※本番 web バンドルに GAP-277 の文字列が無い = Vercel デプロイが main に追随していない</t>
+          <t>[再測 R3] 案件設定の危険な操作 (「プロジェクト削除は 30 日後にハード削除されます。30 日以内であればキャンセル可能。」) から削除 (DELETE 204) → アクティブ一覧から消え「削除済み」タブに「30 日後に完全に削除 / 復元する（残り 30 日）」のカウントダウンつきで出る (GAP-277 の web 側が本番に反映済)。API も deleted_at=2026-09-03T10:46:34Z を記録し GET 詳細は 404。クライアント招待は preview 200→401・発行済みの券で GET /client/projects 401 で無効化。監査 project.delete は復元後 (J38-04) のダッシュボード活動に出る。※付記 (G-14 / 正本に無い観点・別途 QA 用アカウントで再現済): **案件を削除しても、その成果物に発行済みの公開共有リンク (GET /share/{token}) は失効しない** — 案件 DELETE 204 の直後も、さらに WS を DELETE 204 した後も公開 GET は 200 で納品物の本文を返し続けた (410 になるのは所有者が退会したときだけ)。services/outputs/sharing.resolve_share_token が output.deleted_at しか見ておらず、project / workspace の削除を見ていない</t>
         </is>
       </c>
     </row>
@@ -14615,19 +14615,19 @@
           <t>元の状態に戻り、成果物・タスク・コメントが残っている</t>
         </is>
       </c>
-      <c r="K216" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K216" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J38-04-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J38-04-r3.png</t>
         </is>
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 削除済み一覧から復元し元の状態に戻る / 実測: 画面に削除済み一覧・復元導線が無い (UI 復元=null)。API POST /projects/{id}/restore 200 で deleted_at が消え一覧に戻り、タスク 2 件・成果物 3 件・コメント 4 件は残る (データ面は正)。J38-03 の監査 project.delete が dashboard に出る=true ※本番 web バンドルに GAP-277 の文字列が無い = Vercel デプロイが main に追随していない</t>
+          <t>[再測 R3] 「削除済み」タブの「QA jR3 案件 Orion を復元する（残り 30 日）」で復元 (POST /projects/{id}/restore 200) → アクティブ一覧に戻り (deleted_at=null, current_phase=delivery)、タスク 2 件・成果物 2 件・コメント 3 件がそのまま残っている。J38-03 の監査 project.delete もダッシュボードの活動に出る=true</t>
         </is>
       </c>
     </row>
@@ -19066,19 +19066,19 @@
           <t>納品工程が done に遷移し、案件の状態が納品済みとして一覧とダッシュボードに反映される。クライアント側 (J21) に最終版の成果物が見える</t>
         </is>
       </c>
-      <c r="K284" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K284" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J30-15-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J30-15-r3.png</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 納品工程 done・案件が納品済みとして一覧とダッシュボードに反映・クライアントに最終版 / 実測: delivery complete=200 flow delivery=done API current_phase=delivery/delivery/delivery status=draft (API は納品済み=true) / 画面: 一覧カード「のアクティブプロジェクト / 新規プロジェクト / プロジェクトを検索 / すべて / 進行中 / アーカイブ / クライアント案件 / 納品済 / QA jR」 ダッシュボード「プロジェクトダッシュボード / QA jR1 案件 Orion · クライアント案件 · 第 1 段階 ヒアリング中 / 全体進捗率 / 0% / 工程 0/9」 進捗「全体進捗率 / 0% / 工程 0/9 完了 / 未承認 INBOX 件数 / 0 / すべて処理済」 (画面は納品済み=false) / クライアント delivery=true ※本番 web バンドルが main に追随していない (GAP-279 の web 側「進捗カードも flow を優先」未反映の可能性)</t>
+          <t>[再測 R3] (ui3 / ui3b の FAIL 行を上書き) 納品成果物の共有リンクを発行済み (計 2 件・認証なしの公開 GET 200 text/html; charset=utf-8・本文に納品物=true) を確認し、納品工程を確認つきで完了 (confirm なし 403「重要な確認が必要です」/ confirm あり 200) → flow delivery=done。current_phase=delivery が API 詳細・一覧・ダッシュボードで一致 (GAP-279)。画面も 一覧カードに「納品済」バッジ、ダッシュボード「第 10 段階 納品・請求中 / 全体進捗率 100% / 工程 10/10 完了」で納品済みとして反映。クライアント (J21/J23) 側 outputs に delivery v1 が見える。※付記: 一覧カードの工程表記は「工程 9 / 9」でダッシュボードの「工程 10/10」と分母が食い違う (画面間の不一致・正本に無い観点)</t>
         </is>
       </c>
     </row>
@@ -19205,12 +19205,12 @@
       </c>
       <c r="L286" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J23-05-r1.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J23-05-r3.png</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>[再測 R1] 期待: 返信が自分のコメントの下・納品最終版が閲覧できる / 実測: 返信の表示=false、納品成果物の行=true だが「開く」導線=0 個 (content-url 呼出 []) = 画面からは開けない。API 側は GET /client/projects/{pid}/outputs/{oid}/content-url → 200 で実体 200 本文に納品物あり (GAP-268 の API は稼働) ※本番 web バンドルが main に追随しておらず S-L03 の「開く」(GAP-268 web 側) が未反映</t>
+          <t>[再測 R3] (ui4 の行を上書き・より正確に) 期待: 社内の返信が自分のコメントの下に出ている / 納品された最終版の成果物が閲覧できる。実測: **納品成果物は閲覧できる** — S-L03 に「要件定義書 を HTML で開く」「納品書 を HTML で開く」があり、押すと GET /client/projects/{pid}/outputs/{oid}/content-url 200 → 別タブで納品物の本文が開く (GAP-268 の web 側が本番に反映済)。**返信の位置は期待と逆** — 社内の返信「【社内 R3 返信】…」が自分のコメントの **上** に出る (画面の並び ["運営 · QA jR3 改名花子 / 2026/09/03 / 要件","QA クライアント R3 / 2026/09/03 / 要件定義書 "])。原因は API 側 services/client_signin/content.py の list_comments が "order by c.created_at desc" の平坦な一覧を返し、parent_comment_id を返さず画面もスレッド化しないため、返信が「自分のコメントの下」に置かれない。再現: クライアントがコメント → 社内が parent_comment_id つきで返信 → ポータル /portal を開く</t>
         </is>
       </c>
     </row>
@@ -21404,11 +21404,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>43%</t>
         </is>
       </c>
     </row>
@@ -21419,11 +21419,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>7%</t>
         </is>
       </c>
     </row>
@@ -21434,7 +21434,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(正本): GAP-323/324/325 起票、SG01-905 を全書き込み経路の直積に拡張、SG01-907/908 追加、通し R4 再測 (9 行: PASS 6 / FAIL 2 / BLOCKED 1) を集約
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcKo8sr6Bhvy8LEKxeNCsa
</commit_message>
<xml_diff>
--- a/apps/web/.qa/e2e-journey/journey-20260903.xlsx
+++ b/apps/web/.qa/e2e-journey/journey-20260903.xlsx
@@ -8329,19 +8329,19 @@
           <t>選んだ分だけ着手可に遷移し、選んでいないものは変わらない</t>
         </is>
       </c>
-      <c r="K120" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K120" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J48-21-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J48-21-r4.png</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>[再測 R2] 期待: 2 件選んで一括操作で選んだ分だけ着手可 / 実測: S-I01 の選択チェックボックスは着手可のカードにしか無く (準備中カード G/H/I には 0 個、check は 2 件とも不可)、選択バーも出ず、選択バー系の一括「着手可にする」ボタンは無い (画面にあるのはカード単体の「…を着手可にする」6 個 = 1 枚ずつ押すしかない。再実行のハーネスが自分のタイトルの「一括」を含むカード単体ボタンを誤って 1 回押した = E を単体で ready にしただけ)。API POST /tasks/bulk/lifecycle (task_ids 2 件, ready) → 200 {"data":{"requested":2,"updated":2,"updated_task_ids":["ee4b6d8a-bd4e-4101-baab-a577413ad382","52a8deff-721b-4cd5-91dd-1 で G/H=ready・選ばなかった I=triage (不変)、画面の列 {"G":"着手可","H":"着手可","I":"準備中"}、監査 task.bulk_lifecycle ["task.bulk_lifecycle:task:52a8deff","task.bulk_lifecycle:task:ee4b6d8a"] — データ層は正しいが画面から一括着手可はできない (GAP-304 未着手・通し D と同じ)</t>
+          <t>[再測 R4] 準備中カード 3 件のうち 2 件 (G/H) を画面のチェックボックスで選択 → 選択バー「準備中のタスク 2 件を選択中」の「着手可にする2」を押す → POST 200 /tasks/bulk/lifecycle。選んだ G/H だけ ready、選ばなかった I は triage のまま。画面の列 {"G":"着手可","H":"着手可","I":"準備中"}、監査 ["task.bulk_lifecycle:task:e96f3e75","task.bulk_lifecycle:task:e84b7af3"] (GAP-304 解消)</t>
         </is>
       </c>
     </row>
@@ -8591,19 +8591,19 @@
           <t>工程ごとの成果物が一覧に出て、三層がそれぞれ表示された状態になる</t>
         </is>
       </c>
-      <c r="K124" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K124" s="6" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-01-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-01-r4.png</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>[再測 R2] 期待: 工程ごとの成果物が一覧に出て三層 (HTML/JSON/MD) が表示される / 実測: GET /outputs 5 件 (estimate/requirements/verification/hearing)。S-G01 (?output 無し) は「成果物を選択すると表示します」で成果物を選ぶ一覧=0 個。S-F01 工程ごとの成果物欄=["ヒアリング:0件","要件定義:0件","アーキ設計:0件","デザイン:0件","機能分解:0件"] (工程で分かれる=false)。ビューアの表示形式タブ=["HTML"]、HTML 層は iframe 内本文「1. 目的  QA-R2 案件の要件定義書 v1。Nebul」(Mixed Content 0 件)、alert=["この成果物は表形式ではありません。HTML の成果物は本文プレビューで開けます。"]。JSON/MD タブは import 成果物では未生成 (0 個)</t>
+          <t>[再測 R4] 一覧は満たす (GAP-302 解消): S-G01 に「成果物を選ぶ」一覧が 4 行 (stage 毎の最新版 = 見積書v2 / ヒアリングサマリーv1 / 要件定義書v1 / 検証レポートv1) 出て、3 行目を開くと /outputs?output=a7b2adb5-2437-4f33-9a97-f1a456da494e で要件定義書が表示される。S-F01 は工程ごとに中身が変わる: ヒアリング=成果物1(hearing) / 要件定義=成果物1(requirements) / アーキ設計=成果物0 / デザイン=成果物0 / 検証=成果物1(verification) / 納品=成果物0。三層は判定不能 / 理由: 場所=mac — JSON 層 (json_path) と MD 層 (md_path) は AI 実行 (Bridge) が生成するもので、この環境で作れる成果物 (POST /projects/{id}/import) は html_path のみ (対象成果物 json_path=null md_path=null)。そのため S-G01 の表示形式タブは ["HTML"] の 1 層だけ、S-F01 の HTML/JSON/MD も JSON・MD が disabled。解除条件: Mac の Bridge で AI に成果物を生成させ json_path / md_path を持つ成果物で開く</t>
         </is>
       </c>
     </row>
@@ -9518,12 +9518,12 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-16-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-16-r4.png</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>[再測 R2] 画面の「HTML で保存」「Excel で保存」= HTML で保存: HTTP 404 (Authorization 無し) → 遷移先 /outputs/177da0f1-d3ed-4e95-ba54-bd48b80c7b67/export?format=html 「メインコンテンツへスキップ ワークスペース · QA-R2 WS 2026090」 / Excel で保存: HTTP 404 (Authorization 無し) → 遷移先 /outputs/177da0f1-d3ed-4e95-ba54-bd48b80c7b67/export?format=xlsx 「メインコンテンツへスキップ ワークスペース · QA-R2 WS 2026090」。API (Bearer) は html 200 / xlsx 200 (4987 bytes) で得られる。監査 output_downloaded は dashboard に増えず (["task.create:task:9da8b7d4","task.create:task:22fa0df7"]) 観測できない</t>
+          <t>[再測 R4] 期待: ファイルが得られ、監査ログ output_downloaded が記録される / 実測 (ファイル): 画面の「HTML で保存」「Excel で保存」は認証付き fetch (GAP-300) になったが、叩き先が ["WEB オリジン/outputs/a7b2adb5-2437-4f33-9a97-f1a456da494e/export?format=html","WEB オリジン/outputs/a7b2adb5-2437-4f33-9a97-f1a456da494e/export?format=xlsx"] = **API ではなく web オリジン** で 404 (text/html の Next.js 404 ページ) を返し、ダウンロードは発生せず alert「書き出しに失敗しました。時間をおいてもう一度お試しください。」。原因: ShareExportPanel.tsx の apiBase が `process.env.NEXT_PUBLIC_API_URL ?? ""` で、他の全 API 呼び出しが使う lib/auth/connector.ts の API_BASE (未設定なら本番は https://atelier-api-eb.fly.dev) の本番フォールバックを持たないため、Vercel で NEXT_PUBLIC_API_URL 未設定だと相対 URL になる。対照: 同じ成果物に API を Bearer で直接叩くと html 200 544 bytes / xlsx 200 4988 bytes で得られる (API 側は正常)。実測 (監査): dashboard の増分=[] で output_downloaded は記録されず、API 実装 (routes/outputs/__init__.py export_output) にも監査書き込みが無い = 未実装</t>
         </is>
       </c>
     </row>
@@ -9649,12 +9649,12 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-18-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-18-r4.png</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>[再測 R2] 期待: 403 で拒否され成果物は変わらない・閲覧とコメントはできる / 実測: PATCH role=viewer 200。viewer の GET /outputs/{id} 200 (閲覧可)、POST /comments 201 (コメント可) は期待通り。編集系 (各 3 回): POST /sheet [403,403,403]「この操作を行う権限がありません。」(GAP-282 の 500→403 は解消)、POST /share-links [403,403,403]「共有リンクを発行する権限がありません。」(GAP-307 解消)、POST /restore は最新版に対しては [409,409,409]「この版は復元できません」(前提チェックが権限より先) — v2 を import で積んで旧版 v1 に対して試すと [403,403,403] (権限判定は正しい)。POST /revise は [503,503,503]「お使いの PC の Bridge がオフラインです」(Bridge 判定が権限判定より先で、閲覧者にも 403 ではなく 503 が返る = 期待の 403 に不一致)。版数 xlsx 2→2・要件定義 2→3 (増分は対照の owner restore のみ、viewer の操作では不変)。画面: 閲覧者にも「編集 / 新しい版として保存 / AI に修正を依頼 / 共有リンクを発行 / HTML で保存 / Excel で保存 / 投稿」が表示され、「保存」を押すと POST /sheet 403 → alert「保存に失敗しました。」(理由が権限だと分からない)</t>
+          <t>[再測 R4] 期待: 403 で拒否され成果物は変わらない・閲覧とコメントはできる / 実測: PATCH role=viewer 後、viewer の GET /outputs {req,xlsx}=[200,200] (閲覧可)・POST /comments 201・GET /comments 200 (コメント可)。編集系 (各 3 回): sheet [403,403,403] / restore 旧版 v1 [403,403,403] / restore 最新版 v2 [403,403,403] / share-links [403,403,403] / revise [403,403,403] = すべて 403 で、R2 で権限より先に出ていた 503 (revise) と 409 (restore 最新版) は解消 (GAP-311 確認)。画面の「保存」も POST /sheet 403 {detail: この操作を行う権限がありません。} → 画面に「権限がありません。」のトーストが出る (失敗理由が権限だと分かる)。版数 xlsx 1→1・要件定義 2→2 (成果物は不変)、viewer が発行した共有リンク 0 件。**残る不一致 (新規)**: POST /outputs/{id}/ai-file-edit だけ [503,503,503]「お使いの PC の Bridge がオフラインです」で、Bridge 判定が権限判定より先に出る (apps/api/src/routes/outputs/__init__.py の request_output_file_edit に _can_write_output の判定が無い。restore/revise/share-links は line 454/530/683 で判定済み)。閲覧者の画面にも「AI に修正を依頼」ボタンが出ているので実際に踏める経路。GAP-311 と同じ壊れ方が同じ画面の別ボタンに残っている = この 1 点だけで FAIL。併記: 閲覧者の画面に編集系ボタン (編集 / 新しい版として保存 / AI に修正を依頼 / 共有リンクを発行 / 投稿) が出たままなのは GAP-311 が「別途」とした既知事項</t>
         </is>
       </c>
     </row>
@@ -9707,19 +9707,19 @@
           <t>0 件の案内が出る状態になり、エラーにならない</t>
         </is>
       </c>
-      <c r="K141" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K141" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J46-19-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J46-19-r4.png</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>[再測 R2] 期待: 0 件の案内が出てエラーにならない / 実測: GET /outputs=0 件。S-G01 は「成果物を選択すると表示します」(0 件の案内=false)、alert 0 件、API 5xx=0 件、工程画面の成果物欄=「成果物 0 件)」</t>
+          <t>[再測 R4] 成果物 0 件の案件で S-G01 を開くと「この案件にはまだ成果物がありません。工程を進めるかチャットで作成すると、ここに並びます。」と 0 件の案内が出る (GAP-302)。alert 0 件・JS エラー 0 件・API 4xx/5xx 0 件、S-F01 の成果物欄も「成果物 0 件)」でエラーにならない</t>
         </is>
       </c>
     </row>
@@ -12390,19 +12390,19 @@
           <t>日本語のエラーで拒否され、送信履歴に増えない</t>
         </is>
       </c>
-      <c r="K182" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K182" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J47-06-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-06-r4.png</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>[再測 R2] UI: 宛先 'not-an-email' → POST 未送信、アプリのエラー文言=[] (ブラウザ標準の検証のみ: validationMessage「Please include an '@' in the email address. 'not-an-email' is missing an '@'.」= ブラウザ UI 言語依存) / 'foo@' → POST 未送信、アプリのエラー文言=[] (ブラウザ標準の検証のみ: validationMessage「Please enter a part following '@'. 'foo@' is incomplete.」= ブラウザ UI 言語依存); API: 'not-an-email' → 422 "送信内容を確認してください（入力内容: 形式が正しくありません）。"、'foo@' → 422; 送信履歴 1→1 (増えない)</t>
+          <t>[再測 R4] UI: 宛先 'not-an-email' → POST 未送信、アプリのエラー文言=["宛先メールアドレスの形式が正しくありません（例: client@example.com）。"] / 'foo@' → POST 未送信、アプリのエラー文言=["宛先メールアドレスの形式が正しくありません（例: client@example.com）。"]; API: 'not-an-email' → 422 "送信内容を確認してください（入力内容: 形式が正しくありません）。"、'foo@' → 422; 送信履歴 1→1 (増えない)</t>
         </is>
       </c>
     </row>
@@ -12455,19 +12455,19 @@
           <t>一覧から消え、論理削除が記録される。送信履歴は残る</t>
         </is>
       </c>
-      <c r="K183" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K183" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J47-07-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J47-07-r4.png</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>[再測 R2] UI「v2 を削除」→ 確認 → DELETE /sales-docs/{id} 204、一覧 2→1 件・画面から消える、GET detail 404。送信履歴: 削除前 1 件 → 削除後 GET /sales-docs/{id}/sends 404 (ドラフトが不可視になると送信履歴も API/画面から辿れない)。論理削除の監査は運営 API のみで観測不能 (dashboard 増分=["task.update:task:7e00a0ab"])</t>
+          <t>[再測 R4] UI「v2 を削除」→ 確認 → DELETE /sales-docs/{id} 204、一覧 2→1 件・画面から「見積書 Nebula」が消える、GET detail 404。送信履歴: 削除前 1 件 → 削除後も GET /sales-docs/{id}/sends 200 で同じ 1 件が読める (GAP-306 解消。R2 は 404 だった)。論理削除: 削除後に同じ案件・同じ doc_type で新しいドラフトを作ると version=3 が採番される (next_version は deleted_at で絞らない max(version)+1) = 削除した v2 の行が DB に残っている (物理削除ではない)。実装も delete_sales_doc が 'set deleted_at = now()' + AuditWriter(action=sales_doc.delete)。監査行そのものは target_type=workflow_output で、GET /projects/{id}/dashboard の recent_activities (project/task/comment のみ) に出ないため運営 API 無しでは読めない (dashboard 増分=[])</t>
         </is>
       </c>
     </row>
@@ -12520,19 +12520,19 @@
           <t>実行できる種類とコストが一覧に出て、画面表示が GET /cron-actions と一致した状態である</t>
         </is>
       </c>
-      <c r="K184" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K184" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J44-01-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J44-01-r4.png</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>[再測 R2] 期待: 画面表示が GET /cron-actions と一致 / 実測: 6 種中 欠け 6 ["task_replay","knowledge_organize","industry_extract","report_summary","daily_digest","weekly_burndown"]、旧文言残存 ["着手可のタスクを再生する","ナレッジを整理する","横断パターンを抽出する","プラン枠","無料"]</t>
+          <t>[再測 R4] GET /cron-actions 6 種 (task_replay=本人の Claude プラン枠, knowledge_organize=本人の Claude プラン枠/PC接続要, industry_extract=コスト無料, report_summary=本人の Claude プラン枠/PC接続要, daily_digest=コスト無料, weekly_burndown=コスト無料) の title・cost_label・staff・説明が S-O01「2. 何をする？」に全て一致して出る (欠け 0)。API に無い種類カード 0 件、旧ハードコード文言 0 件 (画面の「プラン枠」「無料」は API の cost_label「本人の Claude プラン枠」「コスト無料」の一部)</t>
         </is>
       </c>
     </row>
@@ -17889,19 +17889,19 @@
           <t>入力欄に文章が戻った状態になり、押し直すだけで再送できる</t>
         </is>
       </c>
-      <c r="K266" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K266" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>apps/web/.qa/evidence/shots/journeys/J43-03-r2.png</t>
+          <t>apps/web/.qa/evidence/shots/journeys/J43-03-r4.png</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>[再測 R2] 期待: 入力欄に文章が戻り押し直しで再送 / 実測: 送信 API=POST 200 /chat/threads/3a0342c1-d6b9-467b-a1fc-81c4432c18e8/stream, POST 200 /chat/threads/3a0342c1-d6b9-467b-a1fc-81c4432c18e8/queued/consume、alert=["お使いの PC がまだ接続されていません。設定画面の「Bridge を接続」から接続すると、AI 機能を使えるようになります。"]、入力欄="" (一致=false)、DB messages 1→2、押し直し API=[]</t>
+          <t>[再測 R4] Bridge 未接続 (mode=relay bridge_online=false) で送信 → POST 200 /chat/threads/12a770f1-7dc3-41db-b12b-e7695595ac15/stream, POST 200 /chat/threads/12a770f1-7dc3-41db-b12b-e7695595ac15/queued/consume、画面 alert「お使いのパソコン (Bridge) が未接続のため AI 実行ができません。Bridge アプリを起動してから再送してください。」、入力欄に元の文章がそのまま戻る (一致)、DB の messages は 0→0 件 (応答なしの user 発言を残さない = GAP-310)。送信ボタンは押せる状態 (disabled=false) で、押し直すと再送 (200 /chat/threads/12a770f1-7dc3-41db-b12b-e7695595ac15/stream, 200 /chat/threads/12a770f1-7dc3-41db-b12b-e7695595ac15/queued/consume) され、再び未接続の案内・入力欄に文章が残り DB も 0 件のまま</t>
         </is>
       </c>
     </row>
@@ -21404,11 +21404,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>45%</t>
         </is>
       </c>
     </row>
@@ -21419,11 +21419,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>4%</t>
         </is>
       </c>
     </row>
@@ -21434,7 +21434,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>

</xml_diff>